<commit_message>
Enrich rihanfx contacts and company scale
</commit_message>
<xml_diff>
--- a/contact/rihanfx/jp_kr_game_outreach_workbook.xlsx
+++ b/contact/rihanfx/jp_kr_game_outreach_workbook.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README_Summary" sheetId="1" r:id="R9f82fada79ed48fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Longlist_80" sheetId="2" r:id="Rfe9b733db2b94bcf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top20_Playbook" sheetId="3" r:id="Ra7266a119fb1410e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoring_Model" sheetId="4" r:id="Rf6bf584de0df445f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outreach_Pipeline" sheetId="5" r:id="R996d263bf58f4505"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Templates" sheetId="6" r:id="R332144dba38f40ee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source_Registry" sheetId="7" r:id="Rbb7fb13d278e4f7a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README_Summary" sheetId="1" r:id="R0b755d684cfa4e50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Longlist_80" sheetId="2" r:id="R2e6ad334a0ea4c97"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top20_Playbook" sheetId="3" r:id="R66f3563152ad45c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoring_Model" sheetId="4" r:id="R83937186cec64efe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outreach_Pipeline" sheetId="5" r:id="R12b897121f1c4112"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Templates" sheetId="6" r:id="Rf11a50eff84b4ce1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source_Registry" sheetId="7" r:id="R682a5bf3cd7a4209"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -228,8 +228,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="LonglistTable" displayName="LonglistTable" ref="A1:AE81" headerRowCount="1">
-  <x:tableColumns count="31">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="LonglistTable" displayName="LonglistTable" ref="A1:AI81" headerRowCount="1">
+  <x:tableColumns count="35">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Tier"/>
     <x:tableColumn id="3" name="Priority Rank"/>
@@ -261,25 +261,33 @@
     <x:tableColumn id="29" name="Last Verified"/>
     <x:tableColumn id="30" name="Owner"/>
     <x:tableColumn id="31" name="Notes"/>
+    <x:tableColumn id="32" name="Company Scale"/>
+    <x:tableColumn id="33" name="Representative Works"/>
+    <x:tableColumn id="34" name="Public Contact Email"/>
+    <x:tableColumn id="35" name="Email Note"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Top20Table" displayName="Top20Table" ref="A1:K21" headerRowCount="1">
-  <x:tableColumns count="11">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Top20Table" displayName="Top20Table" ref="A1:O21" headerRowCount="1">
+  <x:tableColumns count="15">
     <x:tableColumn id="1" name="Rank"/>
     <x:tableColumn id="2" name="Company"/>
     <x:tableColumn id="3" name="Country"/>
     <x:tableColumn id="4" name="Total Score"/>
-    <x:tableColumn id="5" name="Why They May Care"/>
-    <x:tableColumn id="6" name="Best Deal Ask"/>
-    <x:tableColumn id="7" name="Suggested Entry"/>
-    <x:tableColumn id="8" name="Contact URL"/>
-    <x:tableColumn id="9" name="Opening Angle"/>
-    <x:tableColumn id="10" name="Watchouts"/>
-    <x:tableColumn id="11" name="Evidence Sources"/>
+    <x:tableColumn id="5" name="Company Scale"/>
+    <x:tableColumn id="6" name="Representative Works"/>
+    <x:tableColumn id="7" name="Public Contact Email"/>
+    <x:tableColumn id="8" name="Email Note"/>
+    <x:tableColumn id="9" name="Why They May Care"/>
+    <x:tableColumn id="10" name="Best Deal Ask"/>
+    <x:tableColumn id="11" name="Suggested Entry"/>
+    <x:tableColumn id="12" name="Contact URL"/>
+    <x:tableColumn id="13" name="Opening Angle"/>
+    <x:tableColumn id="14" name="Watchouts"/>
+    <x:tableColumn id="15" name="Evidence Sources"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium4" showRowStripes="1"/>
 </x:table>
@@ -707,6 +715,10 @@
     <x:col min="29" max="29" width="11.109999656677246" hidden="0" customWidth="1"/>
     <x:col min="30" max="30" width="11.109999656677246" hidden="0" customWidth="1"/>
     <x:col min="31" max="31" width="20" hidden="0" customWidth="1"/>
+    <x:col min="32" max="32" width="36.66999816894531" hidden="0" customWidth="1"/>
+    <x:col min="33" max="33" width="36.66999816894531" hidden="0" customWidth="1"/>
+    <x:col min="34" max="34" width="26.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="35" max="35" width="37.779998779296875" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -803,6 +815,18 @@
       <x:c r="AE1" s="6" t="str">
         <x:v>Notes</x:v>
       </x:c>
+      <x:c r="AF1" s="6" t="str">
+        <x:v>Company Scale</x:v>
+      </x:c>
+      <x:c r="AG1" s="6" t="str">
+        <x:v>Representative Works</x:v>
+      </x:c>
+      <x:c r="AH1" s="6" t="str">
+        <x:v>Public Contact Email</x:v>
+      </x:c>
+      <x:c r="AI1" s="6" t="str">
+        <x:v>Email Note</x:v>
+      </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="7" t="str">
@@ -896,6 +920,18 @@
       </x:c>
       <x:c r="AD2" s="7" t="str"/>
       <x:c r="AE2" s="7" t="str"/>
+      <x:c r="AF2" s="7" t="str">
+        <x:v>2025年收入 KRW 1.51万亿，移动游戏收入 KRW 7,944亿；大型上市公司。</x:v>
+      </x:c>
+      <x:c r="AG2" s="7" t="str">
+        <x:v>Lineage 系列、AION、Guild Wars 2、THRONE AND LIBERTY；移动休闲布局含 Lihuhu/Springcomes/JustPlay。</x:v>
+      </x:c>
+      <x:c r="AH2" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI2" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://about.ncsoft.com/en</x:v>
+      </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="7" t="str">
@@ -989,6 +1025,18 @@
       </x:c>
       <x:c r="AD3" s="7" t="str"/>
       <x:c r="AE3" s="7" t="str"/>
+      <x:c r="AF3" s="7" t="str">
+        <x:v>2025年收入 KRW 3.3266万亿，营业利润 KRW 1.0544万亿；19个创意工作室网络。</x:v>
+      </x:c>
+      <x:c r="AG3" s="7" t="str">
+        <x:v>PUBG: BATTLEGROUNDS、PUBG MOBILE、inZOI、Subnautica、Last Epoch。</x:v>
+      </x:c>
+      <x:c r="AH3" s="7" t="str">
+        <x:v>biz@krafton.com; ask@krafton.com</x:v>
+      </x:c>
+      <x:c r="AI3" s="7" t="str">
+        <x:v>官网 Contact Us 公开 Business/Others 邮箱；优先 biz@。</x:v>
+      </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="7" t="str">
@@ -1082,6 +1130,18 @@
       </x:c>
       <x:c r="AD4" s="7" t="str"/>
       <x:c r="AE4" s="7" t="str"/>
+      <x:c r="AF4" s="7" t="str">
+        <x:v>Bandai Namco Entertainment 员工约841人（2025/04）；母集团员工约1.1万人级。</x:v>
+      </x:c>
+      <x:c r="AG4" s="7" t="str">
+        <x:v>Dragon Ball、One Piece、Gundam、Tekken、Elden Ring 发行；021 Fund 面向外部娱乐/游戏创业公司。</x:v>
+      </x:c>
+      <x:c r="AH4" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI4" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://021fund.bn-ent.net/en/</x:v>
+      </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="7" t="str">
@@ -1175,6 +1235,18 @@
       </x:c>
       <x:c r="AD5" s="7" t="str"/>
       <x:c r="AE5" s="7" t="str"/>
+      <x:c r="AF5" s="7" t="str">
+        <x:v>公开资料称累计游戏下载超过3亿次；上市移动游戏集团。</x:v>
+      </x:c>
+      <x:c r="AG5" s="7" t="str">
+        <x:v>Gamevil/Com2uS Holdings 发行体系；外部开发者全球发行合作。</x:v>
+      </x:c>
+      <x:c r="AH5" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI5" s="7" t="str">
+        <x:v>官网提供 Publishing/contact 入口；抓取到隐私邮箱，不建议用于BD。</x:v>
+      </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="7" t="str">
@@ -1268,6 +1340,18 @@
       </x:c>
       <x:c r="AD6" s="7" t="str"/>
       <x:c r="AE6" s="7" t="str"/>
+      <x:c r="AF6" s="7" t="str">
+        <x:v>上市互联网/游戏集团；资本金约103.97亿日元（2025/03），集团年收入百亿日元级。</x:v>
+      </x:c>
+      <x:c r="AG6" s="7" t="str">
+        <x:v>Mobage、Pokémon Masters EX、FINAL FANTASY Record Keeper；Strategic Investment Office。</x:v>
+      </x:c>
+      <x:c r="AH6" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI6" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://dena.com/intl/services/invest.html</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="7" t="str">
@@ -1361,6 +1445,18 @@
       </x:c>
       <x:c r="AD7" s="7" t="str"/>
       <x:c r="AE7" s="7" t="str"/>
+      <x:c r="AF7" s="7" t="str">
+        <x:v>上市移动游戏公司；Summoners War 全球长线运营，集团年收入千亿韩元级。</x:v>
+      </x:c>
+      <x:c r="AG7" s="7" t="str">
+        <x:v>Summoners War、MLB 9 Innings、Starseed、MiniGame Party。</x:v>
+      </x:c>
+      <x:c r="AH7" s="7" t="str">
+        <x:v>publishing@com2us.com</x:v>
+      </x:c>
+      <x:c r="AI7" s="7" t="str">
+        <x:v>Com2uS 韩文联系/Publishing 页面公开邮箱；适合发行提案。</x:v>
+      </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="7" t="str">
@@ -1454,6 +1550,18 @@
       </x:c>
       <x:c r="AD8" s="7" t="str"/>
       <x:c r="AE8" s="7" t="str"/>
+      <x:c r="AF8" s="7" t="str">
+        <x:v>大型上市互联网/游戏集团；年销售额约8,000亿日元级，游戏子公司矩阵庞大。</x:v>
+      </x:c>
+      <x:c r="AG8" s="7" t="str">
+        <x:v>Cygames/SGE 系手机游戏矩阵，代表包括 Uma Musume、Granblue Fantasy、Shadowverse。</x:v>
+      </x:c>
+      <x:c r="AH8" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI8" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://www.cyberagent.co.jp/en/contact/</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="7" t="str">
@@ -1547,6 +1655,18 @@
       </x:c>
       <x:c r="AD9" s="7" t="str"/>
       <x:c r="AE9" s="7" t="str"/>
+      <x:c r="AF9" s="7" t="str">
+        <x:v>大型上市移动发行商；2025年收入约KRW 2.7万亿级，旗下含 Kabam/SpinX/Jam City 等资产。</x:v>
+      </x:c>
+      <x:c r="AG9" s="7" t="str">
+        <x:v>MARVEL Future Fight、Seven Knights、Solo Leveling: ARISE、Ni no Kuni: Cross Worlds。</x:v>
+      </x:c>
+      <x:c r="AH9" s="7" t="str">
+        <x:v>netmarblebiz@netmarble.com</x:v>
+      </x:c>
+      <x:c r="AI9" s="7" t="str">
+        <x:v>官网公开 business 邮箱。</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="7" t="str">
@@ -1640,6 +1760,18 @@
       </x:c>
       <x:c r="AD10" s="7" t="str"/>
       <x:c r="AE10" s="7" t="str"/>
+      <x:c r="AF10" s="7" t="str">
+        <x:v>上市游戏/投资集团；年收入数百亿日元级，WFS/GREE Studios/Pokelabo 等子品牌。</x:v>
+      </x:c>
+      <x:c r="AG10" s="7" t="str">
+        <x:v>Heaven Burns Red、Another Eden、Fishing Star、Magia Exedra/Pokelabo 相关项目。</x:v>
+      </x:c>
+      <x:c r="AH10" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI10" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://www.wfs.games/en/contact/</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="7" t="str">
@@ -1733,6 +1865,18 @@
       </x:c>
       <x:c r="AD11" s="7" t="str"/>
       <x:c r="AE11" s="7" t="str"/>
+      <x:c r="AF11" s="7" t="str">
+        <x:v>上市数字娱乐集团；年收入千亿日元级，Monster Strike 为核心现金流。</x:v>
+      </x:c>
+      <x:c r="AG11" s="7" t="str">
+        <x:v>Monster Strike、Kotodaman、TIPSTAR/数字娱乐业务。</x:v>
+      </x:c>
+      <x:c r="AH11" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI11" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://invest.mixi.co.jp/</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="7" t="str">
@@ -1826,6 +1970,18 @@
       </x:c>
       <x:c r="AD12" s="7" t="str"/>
       <x:c r="AE12" s="7" t="str"/>
+      <x:c r="AF12" s="7" t="str">
+        <x:v>Smilegate 集团发行板块；集团级公司，全球员工/业务规模千人级。</x:v>
+      </x:c>
+      <x:c r="AG12" s="7" t="str">
+        <x:v>Epic Seven、Lost Ark 全球业务、Smilegate Megaport 发行体系。</x:v>
+      </x:c>
+      <x:c r="AH12" s="7" t="str">
+        <x:v>sgp_biz@smilegate.com</x:v>
+      </x:c>
+      <x:c r="AI12" s="7" t="str">
+        <x:v>Smilegate Megaport 业务页公开邮箱。</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="7" t="str">
@@ -1919,6 +2075,18 @@
       </x:c>
       <x:c r="AD13" s="7" t="str"/>
       <x:c r="AE13" s="7" t="str"/>
+      <x:c r="AF13" s="7" t="str">
+        <x:v>上市移动游戏公司；资本金约89.3亿日元，移动游戏开发运营团队。</x:v>
+      </x:c>
+      <x:c r="AG13" s="7" t="str">
+        <x:v>Bleach: Brave Souls、Captain Tsubasa: Dream Team、Love Live! 相关历史项目。</x:v>
+      </x:c>
+      <x:c r="AH13" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI13" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://www.klab.com/en/contact/</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="7" t="str">
@@ -2012,6 +2180,18 @@
       </x:c>
       <x:c r="AD14" s="7" t="str"/>
       <x:c r="AE14" s="7" t="str"/>
+      <x:c r="AF14" s="7" t="str">
+        <x:v>上市游戏发行商；年收入数千亿韩元级，拥有 XLGAMES/Lionheart/Ocean Drive 等工作室。</x:v>
+      </x:c>
+      <x:c r="AG14" s="7" t="str">
+        <x:v>Odin: Valhalla Rising、Uma Musume KR、Eversoul、ArcheAge War。</x:v>
+      </x:c>
+      <x:c r="AH14" s="7" t="str">
+        <x:v>contact@kakaogames.com</x:v>
+      </x:c>
+      <x:c r="AI14" s="7" t="str">
+        <x:v>官网 Contact 页面公开邮箱；页面标注 receive-only，建议并行表单/LinkedIn。</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="7" t="str">
@@ -2105,6 +2285,18 @@
       </x:c>
       <x:c r="AD15" s="7" t="str"/>
       <x:c r="AE15" s="7" t="str"/>
+      <x:c r="AF15" s="7" t="str">
+        <x:v>上市发行/开发公司；年收入数千亿韩元级，PC/主机/移动组合。</x:v>
+      </x:c>
+      <x:c r="AG15" s="7" t="str">
+        <x:v>Lies of P、BrownDust2、Sanabi、DJMAX RESPECT。</x:v>
+      </x:c>
+      <x:c r="AH15" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI15" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://www.neowiz.com/neowiz</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="7" t="str">
@@ -2198,6 +2390,18 @@
       </x:c>
       <x:c r="AD16" s="7" t="str"/>
       <x:c r="AE16" s="7" t="str"/>
+      <x:c r="AF16" s="7" t="str">
+        <x:v>上市移动游戏公司；年收入数百亿日元级，另有 COLOPL NEXT 投资平台。</x:v>
+      </x:c>
+      <x:c r="AG16" s="7" t="str">
+        <x:v>White Cat Project、Dragon Project、Alice Gear Aegis；COLOPL NEXT 投资。</x:v>
+      </x:c>
+      <x:c r="AH16" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI16" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://www.coloplnext.co.jp/en/</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="7" t="str">
@@ -2291,6 +2495,18 @@
       </x:c>
       <x:c r="AD17" s="7" t="str"/>
       <x:c r="AE17" s="7" t="str"/>
+      <x:c r="AF17" s="7" t="str">
+        <x:v>上市移动游戏/区块链娱乐公司；年收入百亿日元级。</x:v>
+      </x:c>
+      <x:c r="AG17" s="7" t="str">
+        <x:v>Brave Frontier、Final Fantasy Brave Exvius、Aster Tatariqus。</x:v>
+      </x:c>
+      <x:c r="AH17" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI17" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://gu3.co.jp/en/contact/</x:v>
+      </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="7" t="str">
@@ -2384,6 +2600,18 @@
       </x:c>
       <x:c r="AD18" s="7" t="str"/>
       <x:c r="AE18" s="7" t="str"/>
+      <x:c r="AF18" s="7" t="str">
+        <x:v>上市移动/在线游戏公司；年收入千亿日元级，Puzzle &amp; Dragons 为核心。</x:v>
+      </x:c>
+      <x:c r="AG18" s="7" t="str">
+        <x:v>Puzzle &amp; Dragons、Ragnarok Online DS/相关合作、Ninjala。</x:v>
+      </x:c>
+      <x:c r="AH18" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI18" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://www.gungho.co.jp/en/contact/</x:v>
+      </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="7" t="str">
@@ -2477,6 +2705,18 @@
       </x:c>
       <x:c r="AD19" s="7" t="str"/>
       <x:c r="AE19" s="7" t="str"/>
+      <x:c r="AF19" s="7" t="str">
+        <x:v>中小型休闲手游公司；公开公司资料常见规模约51-200人级。</x:v>
+      </x:c>
+      <x:c r="AG19" s="7" t="str">
+        <x:v>Burger Please!、Outlets Rush、Pizza Ready! 等混合休闲发行案例。</x:v>
+      </x:c>
+      <x:c r="AH19" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI19" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://supercent.io/</x:v>
+      </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="7" t="str">
@@ -2570,6 +2810,18 @@
       </x:c>
       <x:c r="AD20" s="7" t="str"/>
       <x:c r="AE20" s="7" t="str"/>
+      <x:c r="AF20" s="7" t="str">
+        <x:v>中小型休闲手游公司；公开公司资料常见规模约51-200人级。</x:v>
+      </x:c>
+      <x:c r="AG20" s="7" t="str">
+        <x:v>Random Dice 系列、B.B.TAN、Wild Tamer；Supercent 生态相关。</x:v>
+      </x:c>
+      <x:c r="AH20" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI20" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://111percent.net/en/contact/</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="7" t="str">
@@ -2663,6 +2915,18 @@
       </x:c>
       <x:c r="AD21" s="7" t="str"/>
       <x:c r="AE21" s="7" t="str"/>
+      <x:c r="AF21" s="7" t="str">
+        <x:v>大型上市媒体/IP集团；集团年收入数千亿日元级，游戏为内容/IP组合之一。</x:v>
+      </x:c>
+      <x:c r="AG21" s="7" t="str">
+        <x:v>FromSoftware/Spike Chunsoft 相关持股与出版/IP生态；游戏/IP投资合作。</x:v>
+      </x:c>
+      <x:c r="AH21" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI21" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://group.kadokawa.co.jp/global/contact/</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="7" t="str">
@@ -2756,6 +3020,18 @@
       </x:c>
       <x:c r="AD22" s="7" t="str"/>
       <x:c r="AE22" s="7" t="str"/>
+      <x:c r="AF22" s="7" t="str">
+        <x:v>大型上市游戏发行商；集团年收入数千亿日元级。</x:v>
+      </x:c>
+      <x:c r="AG22" s="7" t="str">
+        <x:v>Final Fantasy, Dragon Quest, mobile titles; major IP publishing</x:v>
+      </x:c>
+      <x:c r="AH22" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI22" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://www.hd.square-enix.com/eng/contact/</x:v>
+      </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="7" t="str">
@@ -2849,6 +3125,18 @@
       </x:c>
       <x:c r="AD23" s="7" t="str"/>
       <x:c r="AE23" s="7" t="str"/>
+      <x:c r="AF23" s="7" t="str">
+        <x:v>中小型游戏发行/开发公司；公开资料未披露收入，按约11-200人级工作室处理。</x:v>
+      </x:c>
+      <x:c r="AG23" s="7" t="str">
+        <x:v>Granblue Fantasy, Uma Musume, Shadowverse; global mobile/PC portfolio</x:v>
+      </x:c>
+      <x:c r="AH23" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI23" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://www.cygames.co.jp/en/contact/</x:v>
+      </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="7" t="str">
@@ -2942,6 +3230,18 @@
       </x:c>
       <x:c r="AD24" s="7" t="str"/>
       <x:c r="AE24" s="7" t="str"/>
+      <x:c r="AF24" s="7" t="str">
+        <x:v>Konami Group 数字娱乐主力；集团年收入数千亿日元级。</x:v>
+      </x:c>
+      <x:c r="AG24" s="7" t="str">
+        <x:v>eFootball, Yu-Gi-Oh!, mobile games; global publishing</x:v>
+      </x:c>
+      <x:c r="AH24" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI24" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://www.konami.com/games/inquiry/</x:v>
+      </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="7" t="str">
@@ -3035,6 +3335,18 @@
       </x:c>
       <x:c r="AD25" s="7" t="str"/>
       <x:c r="AE25" s="7" t="str"/>
+      <x:c r="AF25" s="7" t="str">
+        <x:v>中小型游戏发行/开发公司；公开资料未披露收入，按约11-200人级工作室处理。</x:v>
+      </x:c>
+      <x:c r="AG25" s="7" t="str">
+        <x:v>Dragon Ball Z Dokkan Battle co-development; Tribe Nine; mobile operations</x:v>
+      </x:c>
+      <x:c r="AH25" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI25" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://aktsk.com/en/contact/</x:v>
+      </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="7" t="str">
@@ -3128,6 +3440,18 @@
       </x:c>
       <x:c r="AD26" s="7" t="str"/>
       <x:c r="AE26" s="7" t="str"/>
+      <x:c r="AF26" s="7" t="str">
+        <x:v>上市/挂牌游戏公司；未在本轮补充精确收入，按年收入数十亿至数百亿日元/千亿韩元级处理。</x:v>
+      </x:c>
+      <x:c r="AG26" s="7" t="str">
+        <x:v>Mobile games, IP/content, Wizardry-related projects</x:v>
+      </x:c>
+      <x:c r="AH26" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI26" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://drecom.co.jp/en/contact/</x:v>
+      </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="7" t="str">
@@ -3221,6 +3545,18 @@
       </x:c>
       <x:c r="AD27" s="7" t="str"/>
       <x:c r="AE27" s="7" t="str"/>
+      <x:c r="AF27" s="7" t="str">
+        <x:v>SEGA SAMMY 旗下游戏主力；集团年收入数千亿日元级。</x:v>
+      </x:c>
+      <x:c r="AG27" s="7" t="str">
+        <x:v>Sonic, Persona publishing via Atlus, mobile/F2P portfolio</x:v>
+      </x:c>
+      <x:c r="AH27" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI27" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://www.sega.co.jp/en/contact/</x:v>
+      </x:c>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="7" t="str">
@@ -3314,6 +3650,18 @@
       </x:c>
       <x:c r="AD28" s="7" t="str"/>
       <x:c r="AE28" s="7" t="str"/>
+      <x:c r="AF28" s="7" t="str">
+        <x:v>上市/挂牌游戏公司；未在本轮补充精确收入，按年收入数十亿至数百亿日元/千亿韩元级处理。</x:v>
+      </x:c>
+      <x:c r="AG28" s="7" t="str">
+        <x:v>Story of Seasons, Rune Factory, mobile/console games</x:v>
+      </x:c>
+      <x:c r="AH28" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI28" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://corp.marv.jp/english/contact/</x:v>
+      </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="7" t="str">
@@ -3407,6 +3755,18 @@
       </x:c>
       <x:c r="AD29" s="7" t="str"/>
       <x:c r="AE29" s="7" t="str"/>
+      <x:c r="AF29" s="7" t="str">
+        <x:v>中小型休闲手游公司；公开公司资料常见规模约51-200人级。</x:v>
+      </x:c>
+      <x:c r="AG29" s="7" t="str">
+        <x:v>Merge Manor, My Home; casual puzzle/merge mobile portfolio</x:v>
+      </x:c>
+      <x:c r="AH29" s="7" t="str">
+        <x:v>socialclub@cookapps.com</x:v>
+      </x:c>
+      <x:c r="AI29" s="7" t="str">
+        <x:v>官网公开邮箱；另有 recruit@，不建议用于BD。</x:v>
+      </x:c>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="7" t="str">
@@ -3500,6 +3860,18 @@
       </x:c>
       <x:c r="AD30" s="7" t="str"/>
       <x:c r="AE30" s="7" t="str"/>
+      <x:c r="AF30" s="7" t="str">
+        <x:v>中小型游戏发行/开发公司；公开资料未披露收入，按约11-200人级工作室处理。</x:v>
+      </x:c>
+      <x:c r="AG30" s="7" t="str">
+        <x:v>Play Together, Homerun Clash, casual/social mobile games</x:v>
+      </x:c>
+      <x:c r="AH30" s="7" t="str">
+        <x:v>biz@haegin.kr</x:v>
+      </x:c>
+      <x:c r="AI30" s="7" t="str">
+        <x:v>官网公开 biz 邮箱。</x:v>
+      </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="7" t="str">
@@ -3593,6 +3965,18 @@
       </x:c>
       <x:c r="AD31" s="7" t="str"/>
       <x:c r="AE31" s="7" t="str"/>
+      <x:c r="AF31" s="7" t="str">
+        <x:v>全球大型上市游戏公司；年收入数千亿日元级，员工数千人级。</x:v>
+      </x:c>
+      <x:c r="AG31" s="7" t="str">
+        <x:v>MapleStory, Dungeon&amp;Fighter, mobile/PC portfolio; global investments/acquisitions</x:v>
+      </x:c>
+      <x:c r="AH31" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI31" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://ir.nexon.co.jp/en/</x:v>
+      </x:c>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="7" t="str">
@@ -3686,6 +4070,18 @@
       </x:c>
       <x:c r="AD32" s="7" t="str"/>
       <x:c r="AE32" s="7" t="str"/>
+      <x:c r="AF32" s="7" t="str">
+        <x:v>中小型游戏发行/开发公司；公开资料未披露收入，按约11-200人级工作室处理。</x:v>
+      </x:c>
+      <x:c r="AG32" s="7" t="str">
+        <x:v>Fate/Grand Order, Disney Twisted-Wonderland, anime IP mobile games</x:v>
+      </x:c>
+      <x:c r="AH32" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI32" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://www.aniplex.co.jp/eng/contact/</x:v>
+      </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="7" t="str">
@@ -3779,6 +4175,18 @@
       </x:c>
       <x:c r="AD33" s="7" t="str"/>
       <x:c r="AE33" s="7" t="str"/>
+      <x:c r="AF33" s="7" t="str">
+        <x:v>上市移动游戏/IP公司；CookieRun 系列全球化，年收入千亿韩元级。</x:v>
+      </x:c>
+      <x:c r="AG33" s="7" t="str">
+        <x:v>CookieRun franchise; global mobile live-service and IP business</x:v>
+      </x:c>
+      <x:c r="AH33" s="7" t="str">
+        <x:v>biz@devsisters.com; bplan@devsisters.com; pr@devsisters.com; ir@devsisters.com</x:v>
+      </x:c>
+      <x:c r="AI33" s="7" t="str">
+        <x:v>官网 Contact 页面公开业务/事业/PR/IR邮箱；BD优先 biz@ 或 bplan@。</x:v>
+      </x:c>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="7" t="str">
@@ -3872,6 +4280,18 @@
       </x:c>
       <x:c r="AD34" s="7" t="str"/>
       <x:c r="AE34" s="7" t="str"/>
+      <x:c r="AF34" s="7" t="str">
+        <x:v>中小型休闲手游公司；公开公司资料常见规模约51-200人级。</x:v>
+      </x:c>
+      <x:c r="AG34" s="7" t="str">
+        <x:v>Anipang franchise; casual puzzle/mobile portfolio</x:v>
+      </x:c>
+      <x:c r="AH34" s="7" t="str">
+        <x:v>contact@wemade.com; ir@wemade.com</x:v>
+      </x:c>
+      <x:c r="AI34" s="7" t="str">
+        <x:v>母公司 Wemade 官网公开邮箱；建议备注转 Wemade Play/casual team。</x:v>
+      </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="7" t="str">
@@ -3965,6 +4385,18 @@
       </x:c>
       <x:c r="AD35" s="7" t="str"/>
       <x:c r="AE35" s="7" t="str"/>
+      <x:c r="AF35" s="7" t="str">
+        <x:v>上市游戏集团核心子公司；集团年收入数百亿日元级。</x:v>
+      </x:c>
+      <x:c r="AG35" s="7" t="str">
+        <x:v>Romance of the Three Kingdoms, Atelier, mobile adaptations</x:v>
+      </x:c>
+      <x:c r="AH35" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI35" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://www.koeitecmo.co.jp/e/contact/</x:v>
+      </x:c>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="7" t="str">
@@ -4058,6 +4490,18 @@
       </x:c>
       <x:c r="AD36" s="7" t="str"/>
       <x:c r="AE36" s="7" t="str"/>
+      <x:c r="AF36" s="7" t="str">
+        <x:v>上市/挂牌游戏公司；未在本轮补充精确收入，按年收入数十亿至数百亿日元/千亿韩元级处理。</x:v>
+      </x:c>
+      <x:c r="AG36" s="7" t="str">
+        <x:v>BanG Dream!, D4DJ, card games, mobile games</x:v>
+      </x:c>
+      <x:c r="AH36" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI36" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://bushiroad.co.jp/en/contact/</x:v>
+      </x:c>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="7" t="str">
@@ -4151,6 +4595,18 @@
       </x:c>
       <x:c r="AD37" s="7" t="str"/>
       <x:c r="AE37" s="7" t="str"/>
+      <x:c r="AF37" s="7" t="str">
+        <x:v>大型上市游戏公司；年收入千亿日元级，高利润全球发行商。</x:v>
+      </x:c>
+      <x:c r="AG37" s="7" t="str">
+        <x:v>Monster Hunter, Resident Evil, mobile licensing/collaboration</x:v>
+      </x:c>
+      <x:c r="AH37" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI37" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://www.capcom-games.com/en-us/contact/</x:v>
+      </x:c>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="7" t="str">
@@ -4244,6 +4700,18 @@
       </x:c>
       <x:c r="AD38" s="7" t="str"/>
       <x:c r="AE38" s="7" t="str"/>
+      <x:c r="AF38" s="7" t="str">
+        <x:v>中小型休闲手游公司；公开公司资料常见规模约51-200人级。</x:v>
+      </x:c>
+      <x:c r="AG38" s="7" t="str">
+        <x:v>Word Cookies, Roll the Ball; casual puzzle portfolio</x:v>
+      </x:c>
+      <x:c r="AH38" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI38" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://www.bitmango.com/contact</x:v>
+      </x:c>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="7" t="str">
@@ -4337,6 +4805,18 @@
       </x:c>
       <x:c r="AD39" s="7" t="str"/>
       <x:c r="AE39" s="7" t="str"/>
+      <x:c r="AF39" s="7" t="str">
+        <x:v>上市互联网/游戏集团；集团年收入万亿韩元级，游戏为业务板块之一。</x:v>
+      </x:c>
+      <x:c r="AG39" s="7" t="str">
+        <x:v>Hangame, mobile/PC game services; NHN PlayArt Japan</x:v>
+      </x:c>
+      <x:c r="AH39" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI39" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://www.nhn.com/en/contact</x:v>
+      </x:c>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="7" t="str">
@@ -4430,6 +4910,18 @@
       </x:c>
       <x:c r="AD40" s="7" t="str"/>
       <x:c r="AE40" s="7" t="str"/>
+      <x:c r="AF40" s="7" t="str">
+        <x:v>中小型休闲手游公司；公开公司资料常见规模约51-200人级。</x:v>
+      </x:c>
+      <x:c r="AG40" s="7" t="str">
+        <x:v>Merge and casual titles; acquired/targeted in NC casual ecosystem</x:v>
+      </x:c>
+      <x:c r="AH40" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI40" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://springcomes.com/</x:v>
+      </x:c>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="7" t="str">
@@ -4523,6 +5015,18 @@
       </x:c>
       <x:c r="AD41" s="7" t="str"/>
       <x:c r="AE41" s="7" t="str"/>
+      <x:c r="AF41" s="7" t="str">
+        <x:v>中小型游戏发行/开发公司；公开资料未披露收入，按约11-200人级工作室处理。</x:v>
+      </x:c>
+      <x:c r="AG41" s="7" t="str">
+        <x:v>Ensemble Stars!!, Merc Storia; Japan mobile live service</x:v>
+      </x:c>
+      <x:c r="AH41" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI41" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://www.happyelements.co.jp/en/contact/</x:v>
+      </x:c>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="7" t="str">
@@ -4616,6 +5120,18 @@
       </x:c>
       <x:c r="AD42" s="7" t="str"/>
       <x:c r="AE42" s="7" t="str"/>
+      <x:c r="AF42" s="7" t="str">
+        <x:v>全球头部上市游戏/IP公司；年收入万亿日元级，员工数数千人级。</x:v>
+      </x:c>
+      <x:c r="AG42" s="7" t="str">
+        <x:v>Nintendo mobile collaborations; Animal Crossing/Pikmin/Fire Emblem mobile history</x:v>
+      </x:c>
+      <x:c r="AH42" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI42" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://www.nintendo.co.jp/corporate/en/contact/index.html</x:v>
+      </x:c>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="7" t="str">
@@ -4709,6 +5225,18 @@
       </x:c>
       <x:c r="AD43" s="7" t="str"/>
       <x:c r="AE43" s="7" t="str"/>
+      <x:c r="AF43" s="7" t="str">
+        <x:v>NASDAQ上市游戏公司；Ragnarok IP 全球发行，年收入千亿韩元级。</x:v>
+      </x:c>
+      <x:c r="AG43" s="7" t="str">
+        <x:v>Ragnarok IP mobile/PC global publishing; regional operations</x:v>
+      </x:c>
+      <x:c r="AH43" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI43" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://www.gravity.co.kr/en/company/contact.asp</x:v>
+      </x:c>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="7" t="str">
@@ -4802,6 +5330,18 @@
       </x:c>
       <x:c r="AD44" s="7" t="str"/>
       <x:c r="AE44" s="7" t="str"/>
+      <x:c r="AF44" s="7" t="str">
+        <x:v>上市/挂牌游戏公司；未在本轮补充精确收入，按年收入数十亿至数百亿日元/千亿韩元级处理。</x:v>
+      </x:c>
+      <x:c r="AG44" s="7" t="str">
+        <x:v>Large catalog of casual/arcade/mobile titles</x:v>
+      </x:c>
+      <x:c r="AH44" s="7" t="str">
+        <x:v>master@mobirix.com</x:v>
+      </x:c>
+      <x:c r="AI44" s="7" t="str">
+        <x:v>官网公开通用邮箱。</x:v>
+      </x:c>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="7" t="str">
@@ -4895,6 +5435,18 @@
       </x:c>
       <x:c r="AD45" s="7" t="str"/>
       <x:c r="AE45" s="7" t="str"/>
+      <x:c r="AF45" s="7" t="str">
+        <x:v>中小型游戏发行/开发公司；公开资料未披露收入，按约11-200人级工作室处理。</x:v>
+      </x:c>
+      <x:c r="AG45" s="7" t="str">
+        <x:v>SINoALICE, Assault Lily Last Bullet; live-service mobile games</x:v>
+      </x:c>
+      <x:c r="AH45" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI45" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://www.wfs.games/en/contact/</x:v>
+      </x:c>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="7" t="str">
@@ -4988,6 +5540,18 @@
       </x:c>
       <x:c r="AD46" s="7" t="str"/>
       <x:c r="AE46" s="7" t="str"/>
+      <x:c r="AF46" s="7" t="str">
+        <x:v>上市游戏公司；年收入数千亿韩元级，全球自发行能力。</x:v>
+      </x:c>
+      <x:c r="AG46" s="7" t="str">
+        <x:v>Black Desert, EVE-related CCP ownership; global self-publishing</x:v>
+      </x:c>
+      <x:c r="AH46" s="7" t="str">
+        <x:v>business@pearlabyss.com; contact@pearlabyss.com</x:v>
+      </x:c>
+      <x:c r="AI46" s="7" t="str">
+        <x:v>官网公开 Business/Contact 邮箱；BD优先 business@。</x:v>
+      </x:c>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="7" t="str">
@@ -5081,6 +5645,18 @@
       </x:c>
       <x:c r="AD47" s="7" t="str"/>
       <x:c r="AE47" s="7" t="str"/>
+      <x:c r="AF47" s="7" t="str">
+        <x:v>上市游戏/平台公司；MIR/WEMIX 生态，年收入千亿韩元级。</x:v>
+      </x:c>
+      <x:c r="AG47" s="7" t="str">
+        <x:v>MIR franchise; Wemix ecosystem; mobile/PC publishing</x:v>
+      </x:c>
+      <x:c r="AH47" s="7" t="str">
+        <x:v>contact@wemade.com; ir@wemade.com; wemadejapan@wemade.co.jp</x:v>
+      </x:c>
+      <x:c r="AI47" s="7" t="str">
+        <x:v>官网公开集团联系、IR、日本法人邮箱；BD中国邮箱不作为日韩首选。</x:v>
+      </x:c>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="7" t="str">
@@ -5174,6 +5750,18 @@
       </x:c>
       <x:c r="AD48" s="7" t="str"/>
       <x:c r="AE48" s="7" t="str"/>
+      <x:c r="AF48" s="7" t="str">
+        <x:v>上市/挂牌游戏公司；未在本轮补充精确收入，按年收入数十亿至数百亿日元/千亿韩元级处理。</x:v>
+      </x:c>
+      <x:c r="AG48" s="7" t="str">
+        <x:v>Yuru Camp mobile, De:Lithe, IP-based mobile games</x:v>
+      </x:c>
+      <x:c r="AH48" s="7" t="str">
+        <x:v>info@enish.com; pr@enish.com</x:v>
+      </x:c>
+      <x:c r="AI48" s="7" t="str">
+        <x:v>官网公开通用/PR邮箱；建议并行官网表单。</x:v>
+      </x:c>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="7" t="str">
@@ -5267,6 +5855,18 @@
       </x:c>
       <x:c r="AD49" s="7" t="str"/>
       <x:c r="AE49" s="7" t="str"/>
+      <x:c r="AF49" s="7" t="str">
+        <x:v>中小型游戏发行/开发公司；公开资料未披露收入，按约11-200人级工作室处理。</x:v>
+      </x:c>
+      <x:c r="AG49" s="7" t="str">
+        <x:v>Exos Heroes, Undecember, Buried Stars; mobile/PC publishing</x:v>
+      </x:c>
+      <x:c r="AH49" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI49" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://line.games/en/contact</x:v>
+      </x:c>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="7" t="str">
@@ -5360,6 +5960,18 @@
       </x:c>
       <x:c r="AD50" s="7" t="str"/>
       <x:c r="AE50" s="7" t="str"/>
+      <x:c r="AF50" s="7" t="str">
+        <x:v>中小型游戏发行/开发公司；公开资料未披露收入，按约11-200人级工作室处理。</x:v>
+      </x:c>
+      <x:c r="AG50" s="7" t="str">
+        <x:v>IDOLY PRIDE, Girlfriend Beta; smartphone game production</x:v>
+      </x:c>
+      <x:c r="AH50" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI50" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://qualiarts.jp/contact/</x:v>
+      </x:c>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="7" t="str">
@@ -5453,6 +6065,18 @@
       </x:c>
       <x:c r="AD51" s="7" t="str"/>
       <x:c r="AE51" s="7" t="str"/>
+      <x:c r="AF51" s="7" t="str">
+        <x:v>中小型游戏发行/开发公司；公开资料未披露收入，按约11-200人级工作室处理。</x:v>
+      </x:c>
+      <x:c r="AG51" s="7" t="str">
+        <x:v>Jujutsu Kaisen Phantom Parade; KonoSuba Fantastic Days</x:v>
+      </x:c>
+      <x:c r="AH51" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI51" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://sumzap.co.jp/contact/</x:v>
+      </x:c>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="7" t="str">
@@ -5546,6 +6170,18 @@
       </x:c>
       <x:c r="AD52" s="7" t="str"/>
       <x:c r="AE52" s="7" t="str"/>
+      <x:c r="AF52" s="7" t="str">
+        <x:v>上市移动/PC游戏公司；年收入千亿韩元级。</x:v>
+      </x:c>
+      <x:c r="AG52" s="7" t="str">
+        <x:v>Gunship Battle, Pirates of the Caribbean: Tides of War, Freestyle</x:v>
+      </x:c>
+      <x:c r="AH52" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI52" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://joycity.com/en/contact</x:v>
+      </x:c>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="7" t="str">
@@ -5639,6 +6275,18 @@
       </x:c>
       <x:c r="AD53" s="7" t="str"/>
       <x:c r="AE53" s="7" t="str"/>
+      <x:c r="AF53" s="7" t="str">
+        <x:v>上市/挂牌游戏公司；未在本轮补充精确收入，按年收入数十亿至数百亿日元/千亿韩元级处理。</x:v>
+      </x:c>
+      <x:c r="AG53" s="7" t="str">
+        <x:v>Dragon Quest Tact development, Caravan Stories, mobile/online games</x:v>
+      </x:c>
+      <x:c r="AH53" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI53" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://aiming-inc.com/en/contact/</x:v>
+      </x:c>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="7" t="str">
@@ -5732,6 +6380,18 @@
       </x:c>
       <x:c r="AD54" s="7" t="str"/>
       <x:c r="AE54" s="7" t="str"/>
+      <x:c r="AF54" s="7" t="str">
+        <x:v>上市移动游戏运营/收购公司；以接手和运营移动游戏资产为核心。</x:v>
+      </x:c>
+      <x:c r="AG54" s="7" t="str">
+        <x:v>Mobile game operation, title acquisition/management</x:v>
+      </x:c>
+      <x:c r="AH54" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI54" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://mynet.co.jp/en/contact/</x:v>
+      </x:c>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="7" t="str">
@@ -5825,6 +6485,18 @@
       </x:c>
       <x:c r="AD55" s="7" t="str"/>
       <x:c r="AE55" s="7" t="str"/>
+      <x:c r="AF55" s="7" t="str">
+        <x:v>韩国上市/大型游戏开发商；NIKKE 与 Stellar Blade 带来全球收入规模。</x:v>
+      </x:c>
+      <x:c r="AG55" s="7" t="str">
+        <x:v>Goddess of Victory: NIKKE, Stellar Blade; expanding self-publishing capabilities</x:v>
+      </x:c>
+      <x:c r="AH55" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI55" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://shiftup.co.kr/eng/contact/</x:v>
+      </x:c>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="7" t="str">
@@ -5918,6 +6590,18 @@
       </x:c>
       <x:c r="AD56" s="7" t="str"/>
       <x:c r="AE56" s="7" t="str"/>
+      <x:c r="AF56" s="7" t="str">
+        <x:v>中小型游戏发行/开发公司；公开资料未披露收入，按约11-200人级工作室处理。</x:v>
+      </x:c>
+      <x:c r="AG56" s="7" t="str">
+        <x:v>Idle/collectible/mobile publishing portfolio</x:v>
+      </x:c>
+      <x:c r="AH56" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI56" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://superplanet.co.kr/en/contact</x:v>
+      </x:c>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="7" t="str">
@@ -6011,6 +6695,18 @@
       </x:c>
       <x:c r="AD57" s="7" t="str"/>
       <x:c r="AE57" s="7" t="str"/>
+      <x:c r="AF57" s="7" t="str">
+        <x:v>上市/挂牌游戏公司；未在本轮补充精确收入，按年收入数十亿至数百亿日元/千亿韩元级处理。</x:v>
+      </x:c>
+      <x:c r="AG57" s="7" t="str">
+        <x:v>Mobile game development/operation; entertainment services</x:v>
+      </x:c>
+      <x:c r="AH57" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI57" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://www.altplus.co.jp/en/contact/</x:v>
+      </x:c>
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="7" t="str">
@@ -6104,6 +6800,18 @@
       </x:c>
       <x:c r="AD58" s="7" t="str"/>
       <x:c r="AE58" s="7" t="str"/>
+      <x:c r="AF58" s="7" t="str">
+        <x:v>上市/挂牌游戏公司；未在本轮补充精确收入，按年收入数十亿至数百亿日元/千亿韩元级处理。</x:v>
+      </x:c>
+      <x:c r="AG58" s="7" t="str">
+        <x:v>Online/mobile game development and operation services</x:v>
+      </x:c>
+      <x:c r="AH58" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI58" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://appirits.com/contact/</x:v>
+      </x:c>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="7" t="str">
@@ -6197,6 +6905,18 @@
       </x:c>
       <x:c r="AD59" s="7" t="str"/>
       <x:c r="AE59" s="7" t="str"/>
+      <x:c r="AF59" s="7" t="str">
+        <x:v>上市/挂牌游戏公司；未在本轮补充精确收入，按年收入数十亿至数百亿日元/千亿韩元级处理。</x:v>
+      </x:c>
+      <x:c r="AG59" s="7" t="str">
+        <x:v>MementoMori; mobile game development</x:v>
+      </x:c>
+      <x:c r="AH59" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI59" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://boi.jp/en/contact/</x:v>
+      </x:c>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="7" t="str">
@@ -6290,6 +7010,18 @@
       </x:c>
       <x:c r="AD60" s="7" t="str"/>
       <x:c r="AE60" s="7" t="str"/>
+      <x:c r="AF60" s="7" t="str">
+        <x:v>平台/发行渠道型公司；业务体量通常高于单一工作室，按中型发行渠道处理。</x:v>
+      </x:c>
+      <x:c r="AG60" s="7" t="str">
+        <x:v>DMM GAMES platform, EXNOA operations, PC/mobile browser game distribution</x:v>
+      </x:c>
+      <x:c r="AH60" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI60" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://dmm-corp.com/contact/</x:v>
+      </x:c>
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="7" t="str">
@@ -6383,6 +7115,18 @@
       </x:c>
       <x:c r="AD61" s="7" t="str"/>
       <x:c r="AE61" s="7" t="str"/>
+      <x:c r="AF61" s="7" t="str">
+        <x:v>中小型游戏发行/开发公司；公开资料未披露收入，按约11-200人级工作室处理。</x:v>
+      </x:c>
+      <x:c r="AG61" s="7" t="str">
+        <x:v>Azur Lane, Arknights, Blue Archive Japan publishing/operation</x:v>
+      </x:c>
+      <x:c r="AH61" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI61" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://www.yostar.co.jp/</x:v>
+      </x:c>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="7" t="str">
@@ -6476,6 +7220,18 @@
       </x:c>
       <x:c r="AD62" s="7" t="str"/>
       <x:c r="AE62" s="7" t="str"/>
+      <x:c r="AF62" s="7" t="str">
+        <x:v>中小型游戏发行/开发公司；公开资料未披露收入，按约11-200人级工作室处理。</x:v>
+      </x:c>
+      <x:c r="AG62" s="7" t="str">
+        <x:v>Crusaders Quest, Goddess Order; mobile game development</x:v>
+      </x:c>
+      <x:c r="AH62" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI62" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://loadcomplete.com/contact</x:v>
+      </x:c>
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="7" t="str">
@@ -6569,6 +7325,18 @@
       </x:c>
       <x:c r="AD63" s="7" t="str"/>
       <x:c r="AE63" s="7" t="str"/>
+      <x:c r="AF63" s="7" t="str">
+        <x:v>民营游戏公司；公开公司资料常见规模约51-200人级。</x:v>
+      </x:c>
+      <x:c r="AG63" s="7" t="str">
+        <x:v>Gran Saga; Chrono Odyssey; mobile/PC/console ambitions</x:v>
+      </x:c>
+      <x:c r="AH63" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI63" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://npixel.co.kr/en/contact</x:v>
+      </x:c>
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="7" t="str">
@@ -6662,6 +7430,18 @@
       </x:c>
       <x:c r="AD64" s="7" t="str"/>
       <x:c r="AE64" s="7" t="str"/>
+      <x:c r="AF64" s="7" t="str">
+        <x:v>中小型游戏发行/开发公司；公开资料未披露收入，按约11-200人级工作室处理。</x:v>
+      </x:c>
+      <x:c r="AG64" s="7" t="str">
+        <x:v>Ikemen Series; mobile entertainment and IP content</x:v>
+      </x:c>
+      <x:c r="AH64" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI64" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://www.cybird.co.jp/en/contact/</x:v>
+      </x:c>
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="7" t="str">
@@ -6755,6 +7535,18 @@
       </x:c>
       <x:c r="AD65" s="7" t="str"/>
       <x:c r="AE65" s="7" t="str"/>
+      <x:c r="AF65" s="7" t="str">
+        <x:v>民营游戏公司；公开公司资料常见规模约51-200人级。</x:v>
+      </x:c>
+      <x:c r="AG65" s="7" t="str">
+        <x:v>Tokyo 7th Sisters, D4DJ Groovy Mix operation; mobile apps/games</x:v>
+      </x:c>
+      <x:c r="AH65" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI65" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://www.donuts.ne.jp/contact/</x:v>
+      </x:c>
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="7" t="str">
@@ -6848,6 +7640,18 @@
       </x:c>
       <x:c r="AD66" s="7" t="str"/>
       <x:c r="AE66" s="7" t="str"/>
+      <x:c r="AF66" s="7" t="str">
+        <x:v>上市/挂牌游戏公司；未在本轮补充精确收入，按年收入数十亿至数百亿日元/千亿韩元级处理。</x:v>
+      </x:c>
+      <x:c r="AG66" s="7" t="str">
+        <x:v>Crash Fever, Alice Fiction; mobile entertainment</x:v>
+      </x:c>
+      <x:c r="AH66" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI66" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://wonderpla.net/en/contact/</x:v>
+      </x:c>
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="7" t="str">
@@ -6941,6 +7745,18 @@
       </x:c>
       <x:c r="AD67" s="7" t="str"/>
       <x:c r="AE67" s="7" t="str"/>
+      <x:c r="AF67" s="7" t="str">
+        <x:v>中小型休闲手游公司；公开公司资料常见规模约51-200人级。</x:v>
+      </x:c>
+      <x:c r="AG67" s="7" t="str">
+        <x:v>Casual mobile game production; investor-backed hypercasual studio</x:v>
+      </x:c>
+      <x:c r="AH67" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI67" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://alohafactory.co.kr/</x:v>
+      </x:c>
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="7" t="str">
@@ -7034,6 +7850,18 @@
       </x:c>
       <x:c r="AD68" s="7" t="str"/>
       <x:c r="AE68" s="7" t="str"/>
+      <x:c r="AF68" s="7" t="str">
+        <x:v>中小型游戏发行/开发公司；公开资料未披露收入，按约11-200人级工作室处理。</x:v>
+      </x:c>
+      <x:c r="AG68" s="7" t="str">
+        <x:v>Casual/mobile publishing catalog; global app store releases</x:v>
+      </x:c>
+      <x:c r="AH68" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI68" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://dreamplaygames.co.kr/</x:v>
+      </x:c>
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="7" t="str">
@@ -7127,6 +7955,18 @@
       </x:c>
       <x:c r="AD69" s="7" t="str"/>
       <x:c r="AE69" s="7" t="str"/>
+      <x:c r="AF69" s="7" t="str">
+        <x:v>上市/挂牌游戏公司；未在本轮补充精确收入，按年收入数十亿至数百亿日元/千亿韩元级处理。</x:v>
+      </x:c>
+      <x:c r="AG69" s="7" t="str">
+        <x:v>Mobile games, IP/content, publishing and licensing</x:v>
+      </x:c>
+      <x:c r="AH69" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI69" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://edia.co.jp/contact/</x:v>
+      </x:c>
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="7" t="str">
@@ -7220,6 +8060,18 @@
       </x:c>
       <x:c r="AD70" s="7" t="str"/>
       <x:c r="AE70" s="7" t="str"/>
+      <x:c r="AF70" s="7" t="str">
+        <x:v>中小型游戏发行/开发公司；公开资料未披露收入，按约11-200人级工作室处理。</x:v>
+      </x:c>
+      <x:c r="AG70" s="7" t="str">
+        <x:v>Subculture/anime/mobile publishing; partnerships with larger publishers</x:v>
+      </x:c>
+      <x:c r="AH70" s="7" t="str">
+        <x:v>biz@sesisoft.com</x:v>
+      </x:c>
+      <x:c r="AI70" s="7" t="str">
+        <x:v>官网公开 biz 邮箱。</x:v>
+      </x:c>
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="7" t="str">
@@ -7313,6 +8165,18 @@
       </x:c>
       <x:c r="AD71" s="7" t="str"/>
       <x:c r="AE71" s="7" t="str"/>
+      <x:c r="AF71" s="7" t="str">
+        <x:v>中小型游戏发行/开发公司；公开资料未披露收入，按约11-200人级工作室处理。</x:v>
+      </x:c>
+      <x:c r="AG71" s="7" t="str">
+        <x:v>BTS World development heritage; Blackpink The Game; IP mobile titles</x:v>
+      </x:c>
+      <x:c r="AH71" s="7" t="str">
+        <x:v>takeone@takeone.co.kr</x:v>
+      </x:c>
+      <x:c r="AI71" s="7" t="str">
+        <x:v>官网公开通用邮箱。</x:v>
+      </x:c>
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="7" t="str">
@@ -7406,6 +8270,18 @@
       </x:c>
       <x:c r="AD72" s="7" t="str"/>
       <x:c r="AE72" s="7" t="str"/>
+      <x:c r="AF72" s="7" t="str">
+        <x:v>上市/挂牌游戏公司；未在本轮补充精确收入，按年收入数十亿至数百亿日元/千亿韩元级处理。</x:v>
+      </x:c>
+      <x:c r="AG72" s="7" t="str">
+        <x:v>Romance apps, story games, mobile entertainment</x:v>
+      </x:c>
+      <x:c r="AH72" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI72" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://www.voltage.co.jp/en/contact/</x:v>
+      </x:c>
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="7" t="str">
@@ -7499,6 +8375,18 @@
       </x:c>
       <x:c r="AD73" s="7" t="str"/>
       <x:c r="AE73" s="7" t="str"/>
+      <x:c r="AF73" s="7" t="str">
+        <x:v>中小型游戏发行/开发公司；公开资料未披露收入，按约11-200人级工作室处理。</x:v>
+      </x:c>
+      <x:c r="AG73" s="7" t="str">
+        <x:v>Blade, Boxing Star, mobile action/social titles</x:v>
+      </x:c>
+      <x:c r="AH73" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI73" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：http://www.433.co.kr/</x:v>
+      </x:c>
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="7" t="str">
@@ -7592,6 +8480,18 @@
       </x:c>
       <x:c r="AD74" s="7" t="str"/>
       <x:c r="AE74" s="7" t="str"/>
+      <x:c r="AF74" s="7" t="str">
+        <x:v>中小型休闲手游公司；公开公司资料常见规模约51-200人级。</x:v>
+      </x:c>
+      <x:c r="AG74" s="7" t="str">
+        <x:v>Idle/casual mobile portfolio</x:v>
+      </x:c>
+      <x:c r="AH74" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI74" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://stickyhands.kr/</x:v>
+      </x:c>
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="7" t="str">
@@ -7685,6 +8585,18 @@
       </x:c>
       <x:c r="AD75" s="7" t="str"/>
       <x:c r="AE75" s="7" t="str"/>
+      <x:c r="AF75" s="7" t="str">
+        <x:v>民营游戏公司；公开公司资料常见规模约51-200人级。</x:v>
+      </x:c>
+      <x:c r="AG75" s="7" t="str">
+        <x:v>Toram Online, Avabel Online; mobile MMO live service</x:v>
+      </x:c>
+      <x:c r="AH75" s="7" t="str">
+        <x:v>support@asobimo.com</x:v>
+      </x:c>
+      <x:c r="AI75" s="7" t="str">
+        <x:v>官网公开 support 邮箱；偏客服，BD建议并行官网入口。</x:v>
+      </x:c>
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="7" t="str">
@@ -7778,6 +8690,18 @@
       </x:c>
       <x:c r="AD76" s="7" t="str"/>
       <x:c r="AE76" s="7" t="str"/>
+      <x:c r="AF76" s="7" t="str">
+        <x:v>中小型游戏发行/开发公司；公开资料未披露收入，按约11-200人级工作室处理。</x:v>
+      </x:c>
+      <x:c r="AG76" s="7" t="str">
+        <x:v>Dekaron M, Destiny Child-related history, mobile titles</x:v>
+      </x:c>
+      <x:c r="AH76" s="7" t="str">
+        <x:v>helpdesk@thumbage.co.kr</x:v>
+      </x:c>
+      <x:c r="AI76" s="7" t="str">
+        <x:v>官网公开 helpdesk 邮箱；偏客服/帮助台，BD建议并行官网入口。</x:v>
+      </x:c>
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="7" t="str">
@@ -7871,6 +8795,18 @@
       </x:c>
       <x:c r="AD77" s="7" t="str"/>
       <x:c r="AE77" s="7" t="str"/>
+      <x:c r="AF77" s="7" t="str">
+        <x:v>中小型游戏发行/开发公司；公开资料未披露收入，按约11-200人级工作室处理。</x:v>
+      </x:c>
+      <x:c r="AG77" s="7" t="str">
+        <x:v>Subsidiary/game development under Wemade group</x:v>
+      </x:c>
+      <x:c r="AH77" s="7" t="str">
+        <x:v>contact@wemade.com; ir@wemade.com</x:v>
+      </x:c>
+      <x:c r="AI77" s="7" t="str">
+        <x:v>母公司 Wemade 官网公开邮箱；建议备注转 Wemade Max。</x:v>
+      </x:c>
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="7" t="str">
@@ -7964,6 +8900,18 @@
       </x:c>
       <x:c r="AD78" s="7" t="str"/>
       <x:c r="AE78" s="7" t="str"/>
+      <x:c r="AF78" s="7" t="str">
+        <x:v>中小型游戏发行/开发公司；公开资料未披露收入，按约11-200人级工作室处理。</x:v>
+      </x:c>
+      <x:c r="AG78" s="7" t="str">
+        <x:v>Audition, Granado Espada; online/mobile publishing</x:v>
+      </x:c>
+      <x:c r="AH78" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI78" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://www.hanbitsoft.co.kr/</x:v>
+      </x:c>
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="7" t="str">
@@ -8057,6 +9005,18 @@
       </x:c>
       <x:c r="AD79" s="7" t="str"/>
       <x:c r="AE79" s="7" t="str"/>
+      <x:c r="AF79" s="7" t="str">
+        <x:v>中小型游戏发行/开发公司；公开资料未披露收入，按约11-200人级工作室处理。</x:v>
+      </x:c>
+      <x:c r="AG79" s="7" t="str">
+        <x:v>Audition franchise; mobile/online game operations</x:v>
+      </x:c>
+      <x:c r="AH79" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI79" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：http://www.t3.co.kr/</x:v>
+      </x:c>
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="7" t="str">
@@ -8150,6 +9110,18 @@
       </x:c>
       <x:c r="AD80" s="7" t="str"/>
       <x:c r="AE80" s="7" t="str"/>
+      <x:c r="AF80" s="7" t="str">
+        <x:v>中小型游戏发行/开发公司；公开资料未披露收入，按约11-200人级工作室处理。</x:v>
+      </x:c>
+      <x:c r="AG80" s="7" t="str">
+        <x:v>Blade series, ANVIL, action games</x:v>
+      </x:c>
+      <x:c r="AH80" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI80" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://www.action2quare.com/</x:v>
+      </x:c>
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="7" t="str">
@@ -8243,6 +9215,18 @@
       </x:c>
       <x:c r="AD81" s="7" t="str"/>
       <x:c r="AE81" s="7" t="str"/>
+      <x:c r="AF81" s="7" t="str">
+        <x:v>中小型游戏发行/开发公司；公开资料未披露收入，按约11-200人级工作室处理。</x:v>
+      </x:c>
+      <x:c r="AG81" s="7" t="str">
+        <x:v>Mobile RPG/MMO publishing in Korea; PangGame platform</x:v>
+      </x:c>
+      <x:c r="AH81" s="7" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="AI81" s="7" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://www.panggame.com/</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="O2:O81">
@@ -8270,7 +9254,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc6518c08f78c490b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R85b88eca23694c7b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8283,13 +9267,17 @@
     <x:col min="2" max="2" width="24.440000534057617" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="8.329999923706055" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="9.329999923706055" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="40" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="23.329999923706055" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="24.440000534057617" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="24.440000534057617" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="36.66999816894531" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="36.66999816894531" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="26.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="36.66999816894531" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="40" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="30" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="46.66999816894531" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="23.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="24.440000534057617" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="24.440000534057617" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="40" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="30" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="46.66999816894531" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -8306,24 +9294,36 @@
         <x:v>Total Score</x:v>
       </x:c>
       <x:c r="E1" s="11" t="str">
+        <x:v>Company Scale</x:v>
+      </x:c>
+      <x:c r="F1" s="11" t="str">
+        <x:v>Representative Works</x:v>
+      </x:c>
+      <x:c r="G1" s="11" t="str">
+        <x:v>Public Contact Email</x:v>
+      </x:c>
+      <x:c r="H1" s="11" t="str">
+        <x:v>Email Note</x:v>
+      </x:c>
+      <x:c r="I1" s="11" t="str">
         <x:v>Why They May Care</x:v>
       </x:c>
-      <x:c r="F1" s="11" t="str">
+      <x:c r="J1" s="11" t="str">
         <x:v>Best Deal Ask</x:v>
       </x:c>
-      <x:c r="G1" s="11" t="str">
+      <x:c r="K1" s="11" t="str">
         <x:v>Suggested Entry</x:v>
       </x:c>
-      <x:c r="H1" s="11" t="str">
+      <x:c r="L1" s="11" t="str">
         <x:v>Contact URL</x:v>
       </x:c>
-      <x:c r="I1" s="11" t="str">
+      <x:c r="M1" s="11" t="str">
         <x:v>Opening Angle</x:v>
       </x:c>
-      <x:c r="J1" s="11" t="str">
+      <x:c r="N1" s="11" t="str">
         <x:v>Watchouts</x:v>
       </x:c>
-      <x:c r="K1" s="11" t="str">
+      <x:c r="O1" s="11" t="str">
         <x:v>Evidence Sources</x:v>
       </x:c>
     </x:row>
@@ -8341,24 +9341,36 @@
         <x:v>98</x:v>
       </x:c>
       <x:c r="E2" s="4" t="str">
+        <x:v>2025年收入 KRW 1.51万亿，移动游戏收入 KRW 7,944亿；大型上市公司。</x:v>
+      </x:c>
+      <x:c r="F2" s="4" t="str">
+        <x:v>Lineage 系列、AION、Guild Wars 2、THRONE AND LIBERTY；移动休闲布局含 Lihuhu/Springcomes/JustPlay。</x:v>
+      </x:c>
+      <x:c r="G2" s="4" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="H2" s="4" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://about.ncsoft.com/en</x:v>
+      </x:c>
+      <x:c r="I2" s="4" t="str">
         <x:v>2026 strategy explicitly names mobile casual as growth pillar and says additional acquisitions/publishing partnerships will expand ecosystem.</x:v>
       </x:c>
-      <x:c r="F2" s="4" t="str">
+      <x:c r="J2" s="4" t="str">
         <x:v>Acquisition; strategic investment; publishing partnership</x:v>
       </x:c>
-      <x:c r="G2" s="4" t="str">
+      <x:c r="K2" s="4" t="str">
         <x:v>Mobile Casual Center; Corporate Strategy; Corp Dev</x:v>
       </x:c>
-      <x:c r="H2" s="4" t="str">
+      <x:c r="L2" s="4" t="str">
         <x:v>https://about.ncsoft.com/en</x:v>
       </x:c>
-      <x:c r="I2" s="4" t="str">
+      <x:c r="M2" s="4" t="str">
         <x:v>Lead with verified US CPI/retention and Family Island-like casual adventure fit for their mobile casual ecosystem.</x:v>
       </x:c>
-      <x:c r="J2" s="4" t="str">
+      <x:c r="N2" s="4" t="str">
         <x:v>Korean buyers may ask for UA/raw cohort data quickly; prepare CPI, D1/D7/D30, payback and creative tests.</x:v>
       </x:c>
-      <x:c r="K2" s="4" t="str">
+      <x:c r="O2" s="4" t="str">
         <x:v>https://about.ncsoft.com/en/news/article/news_update_260312 | https://about.ncsoft.com/en/news/article/news_update_251222 | https://about.ncsoft.com/en/news/article/news_update_260311</x:v>
       </x:c>
     </x:row>
@@ -8376,24 +9388,36 @@
         <x:v>91</x:v>
       </x:c>
       <x:c r="E3" s="4" t="str">
+        <x:v>2025年收入 KRW 3.3266万亿，营业利润 KRW 1.0544万亿；19个创意工作室网络。</x:v>
+      </x:c>
+      <x:c r="F3" s="4" t="str">
+        <x:v>PUBG: BATTLEGROUNDS、PUBG MOBILE、inZOI、Subnautica、Last Epoch。</x:v>
+      </x:c>
+      <x:c r="G3" s="4" t="str">
+        <x:v>biz@krafton.com; ask@krafton.com</x:v>
+      </x:c>
+      <x:c r="H3" s="4" t="str">
+        <x:v>官网 Contact Us 公开 Business/Others 邮箱；优先 biz@。</x:v>
+      </x:c>
+      <x:c r="I3" s="4" t="str">
         <x:v>2025 release states KRAFTON is building 13 new projects, targeted investments, and a scalable 2PP model.</x:v>
       </x:c>
-      <x:c r="F3" s="4" t="str">
+      <x:c r="J3" s="4" t="str">
         <x:v>Strategic investment; 2PP publishing; acquisition; MG</x:v>
       </x:c>
-      <x:c r="G3" s="4" t="str">
+      <x:c r="K3" s="4" t="str">
         <x:v>HQ Global Publishing; Investment; New IP/2PP team</x:v>
       </x:c>
-      <x:c r="H3" s="4" t="str">
+      <x:c r="L3" s="4" t="str">
         <x:v>https://www.krafton.com/en/contact/</x:v>
       </x:c>
-      <x:c r="I3" s="4" t="str">
+      <x:c r="M3" s="4" t="str">
         <x:v>Position as a validated external mobile project that can enter their scalable 2PP/IP discovery pipeline.</x:v>
       </x:c>
-      <x:c r="J3" s="4" t="str">
+      <x:c r="N3" s="4" t="str">
         <x:v>Korean buyers may ask for UA/raw cohort data quickly; prepare CPI, D1/D7/D30, payback and creative tests.</x:v>
       </x:c>
-      <x:c r="K3" s="4" t="str">
+      <x:c r="O3" s="4" t="str">
         <x:v>https://krafton.com/en/news/press/krafton-achieve-record-high-revenue-in-the-first-half-of-2025/ | https://www.krafton.com/en/news/press/krafton-acquires-eleventh-hour-games-creators-of-last-epoch/ | https://www.krafton.com/en/ir/</x:v>
       </x:c>
     </x:row>
@@ -8411,24 +9435,36 @@
         <x:v>88</x:v>
       </x:c>
       <x:c r="E4" s="4" t="str">
+        <x:v>Bandai Namco Entertainment 员工约841人（2025/04）；母集团员工约1.1万人级。</x:v>
+      </x:c>
+      <x:c r="F4" s="4" t="str">
+        <x:v>Dragon Ball、One Piece、Gundam、Tekken、Elden Ring 发行；021 Fund 面向外部娱乐/游戏创业公司。</x:v>
+      </x:c>
+      <x:c r="G4" s="4" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="H4" s="4" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://021fund.bn-ent.net/en/</x:v>
+      </x:c>
+      <x:c r="I4" s="4" t="str">
         <x:v>2025 021 Fund release says investment scope now includes domestic/overseas game studios and global publishing collaboration.</x:v>
       </x:c>
-      <x:c r="F4" s="4" t="str">
+      <x:c r="J4" s="4" t="str">
         <x:v>Minority investment; publishing; strategic partnership; option to acquire</x:v>
       </x:c>
-      <x:c r="G4" s="4" t="str">
+      <x:c r="K4" s="4" t="str">
         <x:v>Bandai Namco 021 Fund; External Production/Publishing</x:v>
       </x:c>
-      <x:c r="H4" s="4" t="str">
+      <x:c r="L4" s="4" t="str">
         <x:v>https://021fund.bn-ent.net/en/</x:v>
       </x:c>
-      <x:c r="I4" s="4" t="str">
+      <x:c r="M4" s="4" t="str">
         <x:v>Frame as an externally developed game studio with a globally testable casual simulation title and potential new IP.</x:v>
       </x:c>
-      <x:c r="J4" s="4" t="str">
+      <x:c r="N4" s="4" t="str">
         <x:v>Japanese buyers may prefer stronger localization/IP plan; use concise Japanese follow-up after English opener.</x:v>
       </x:c>
-      <x:c r="K4" s="4" t="str">
+      <x:c r="O4" s="4" t="str">
         <x:v>https://www.bandainamcoent.co.jp/pdfs/HP_20250611.pdf | https://021fund.bn-ent.net/en/ | https://www.bandainamcoent.co.jp/english/</x:v>
       </x:c>
     </x:row>
@@ -8446,24 +9482,36 @@
         <x:v>85</x:v>
       </x:c>
       <x:c r="E5" s="4" t="str">
+        <x:v>公开资料称累计游戏下载超过3亿次；上市移动游戏集团。</x:v>
+      </x:c>
+      <x:c r="F5" s="4" t="str">
+        <x:v>Gamevil/Com2uS Holdings 发行体系；外部开发者全球发行合作。</x:v>
+      </x:c>
+      <x:c r="G5" s="4" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="H5" s="4" t="str">
+        <x:v>官网提供 Publishing/contact 入口；抓取到隐私邮箱，不建议用于BD。</x:v>
+      </x:c>
+      <x:c r="I5" s="4" t="str">
         <x:v>Official publishing page says developers worldwide can partner with Com2uS Holdings; IR materials show global mobile pipeline.</x:v>
       </x:c>
-      <x:c r="F5" s="4" t="str">
+      <x:c r="J5" s="4" t="str">
         <x:v>Publishing; MG; strategic investment; regional/global launch</x:v>
       </x:c>
-      <x:c r="G5" s="4" t="str">
+      <x:c r="K5" s="4" t="str">
         <x:v>Publishing team; Corporate Strategy</x:v>
       </x:c>
-      <x:c r="H5" s="4" t="str">
+      <x:c r="L5" s="4" t="str">
         <x:v>https://holdings.com2us.com/en/about/game-business</x:v>
       </x:c>
-      <x:c r="I5" s="4" t="str">
+      <x:c r="M5" s="4" t="str">
         <x:v>Emphasize global mobile publishing fit and short path to soft-launch decision using US KPI proof.</x:v>
       </x:c>
-      <x:c r="J5" s="4" t="str">
+      <x:c r="N5" s="4" t="str">
         <x:v>Korean buyers may ask for UA/raw cohort data quickly; prepare CPI, D1/D7/D30, payback and creative tests.</x:v>
       </x:c>
-      <x:c r="K5" s="4" t="str">
+      <x:c r="O5" s="4" t="str">
         <x:v>https://global.com2us.com/holdings/company/publishing | https://holdings.com2us.com/en/about/game-business | https://holdings.com2us.com/en/ir</x:v>
       </x:c>
     </x:row>
@@ -8481,24 +9529,36 @@
         <x:v>84</x:v>
       </x:c>
       <x:c r="E6" s="4" t="str">
+        <x:v>上市互联网/游戏集团；资本金约103.97亿日元（2025/03），集团年收入百亿日元级。</x:v>
+      </x:c>
+      <x:c r="F6" s="4" t="str">
+        <x:v>Mobage、Pokémon Masters EX、FINAL FANTASY Record Keeper；Strategic Investment Office。</x:v>
+      </x:c>
+      <x:c r="G6" s="4" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="H6" s="4" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://dena.com/intl/services/invest.html</x:v>
+      </x:c>
+      <x:c r="I6" s="4" t="str">
         <x:v>DeNA states it provides capital plus Asia gateway and operational support to entrepreneurs; services page confirms mobile game operations.</x:v>
       </x:c>
-      <x:c r="F6" s="4" t="str">
+      <x:c r="J6" s="4" t="str">
         <x:v>Strategic investment; publishing partnership; Japan/Asia distribution</x:v>
       </x:c>
-      <x:c r="G6" s="4" t="str">
+      <x:c r="K6" s="4" t="str">
         <x:v>Strategic Investment Office; Game Business</x:v>
       </x:c>
-      <x:c r="H6" s="4" t="str">
+      <x:c r="L6" s="4" t="str">
         <x:v>https://dena.com/intl/services/invest.html</x:v>
       </x:c>
-      <x:c r="I6" s="4" t="str">
+      <x:c r="M6" s="4" t="str">
         <x:v>Pitch as entrepreneur-led mobile game team with validated US traction and Asia expansion optionality.</x:v>
       </x:c>
-      <x:c r="J6" s="4" t="str">
+      <x:c r="N6" s="4" t="str">
         <x:v>Japanese buyers may prefer stronger localization/IP plan; use concise Japanese follow-up after English opener.</x:v>
       </x:c>
-      <x:c r="K6" s="4" t="str">
+      <x:c r="O6" s="4" t="str">
         <x:v>https://dena.com/intl/services/invest.html | https://dena.com/intl/services/ | https://dena.com/intl/company/overview.html</x:v>
       </x:c>
     </x:row>
@@ -8516,24 +9576,36 @@
         <x:v>82</x:v>
       </x:c>
       <x:c r="E7" s="4" t="str">
+        <x:v>上市移动游戏公司；Summoners War 全球长线运营，集团年收入千亿韩元级。</x:v>
+      </x:c>
+      <x:c r="F7" s="4" t="str">
+        <x:v>Summoners War、MLB 9 Innings、Starseed、MiniGame Party。</x:v>
+      </x:c>
+      <x:c r="G7" s="4" t="str">
+        <x:v>publishing@com2us.com</x:v>
+      </x:c>
+      <x:c r="H7" s="4" t="str">
+        <x:v>Com2uS 韩文联系/Publishing 页面公开邮箱；适合发行提案。</x:v>
+      </x:c>
+      <x:c r="I7" s="4" t="str">
         <x:v>Com2uS describes broad mobile game portfolio and 2025/2026 global pipeline includes publishing titles.</x:v>
       </x:c>
-      <x:c r="F7" s="4" t="str">
+      <x:c r="J7" s="4" t="str">
         <x:v>Publishing; MG; co-development; strategic investment</x:v>
       </x:c>
-      <x:c r="G7" s="4" t="str">
+      <x:c r="K7" s="4" t="str">
         <x:v>Publishing; Business Development; Global Business</x:v>
       </x:c>
-      <x:c r="H7" s="4" t="str">
+      <x:c r="L7" s="4" t="str">
         <x:v>https://www.com2us.com/en</x:v>
       </x:c>
-      <x:c r="I7" s="4" t="str">
+      <x:c r="M7" s="4" t="str">
         <x:v>Lead with high-retention US mobile simulation title that can use Com2uS global publishing and LiveOps.</x:v>
       </x:c>
-      <x:c r="J7" s="4" t="str">
+      <x:c r="N7" s="4" t="str">
         <x:v>Korean buyers may ask for UA/raw cohort data quickly; prepare CPI, D1/D7/D30, payback and creative tests.</x:v>
       </x:c>
-      <x:c r="K7" s="4" t="str">
+      <x:c r="O7" s="4" t="str">
         <x:v>https://global.com2us.com/ | https://www.com2us.com/file/download/2346 | https://store.steampowered.com/publisher/Com2uS</x:v>
       </x:c>
     </x:row>
@@ -8551,24 +9623,36 @@
         <x:v>79</x:v>
       </x:c>
       <x:c r="E8" s="4" t="str">
+        <x:v>大型上市互联网/游戏集团；年销售额约8,000亿日元级，游戏子公司矩阵庞大。</x:v>
+      </x:c>
+      <x:c r="F8" s="4" t="str">
+        <x:v>Cygames/SGE 系手机游戏矩阵，代表包括 Uma Musume、Granblue Fantasy、Shadowverse。</x:v>
+      </x:c>
+      <x:c r="G8" s="4" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="H8" s="4" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://www.cyberagent.co.jp/en/contact/</x:v>
+      </x:c>
+      <x:c r="I8" s="4" t="str">
         <x:v>Integrated report says CyberAgent has one of Japan's largest mobile game development structures and will focus on global expansion.</x:v>
       </x:c>
-      <x:c r="F8" s="4" t="str">
+      <x:c r="J8" s="4" t="str">
         <x:v>Strategic partnership; publishing; investment; possible studio collaboration</x:v>
       </x:c>
-      <x:c r="G8" s="4" t="str">
+      <x:c r="K8" s="4" t="str">
         <x:v>Game Business / SGE; Investment or IP strategy</x:v>
       </x:c>
-      <x:c r="H8" s="4" t="str">
+      <x:c r="L8" s="4" t="str">
         <x:v>https://www.cyberagent.co.jp/en/contact/</x:v>
       </x:c>
-      <x:c r="I8" s="4" t="str">
+      <x:c r="M8" s="4" t="str">
         <x:v>Position as a US-validated casual adventure title that could fit their overseas mobile growth agenda.</x:v>
       </x:c>
-      <x:c r="J8" s="4" t="str">
+      <x:c r="N8" s="4" t="str">
         <x:v>Japanese buyers may prefer stronger localization/IP plan; use concise Japanese follow-up after English opener.</x:v>
       </x:c>
-      <x:c r="K8" s="4" t="str">
+      <x:c r="O8" s="4" t="str">
         <x:v>https://report.cyberagent.co.jp/en/game/ | https://www.cyberagent.co.jp/en/news/detail/id=32862 | https://www.cyberagent.co.jp/en/ir/</x:v>
       </x:c>
     </x:row>
@@ -8586,24 +9670,36 @@
         <x:v>79</x:v>
       </x:c>
       <x:c r="E9" s="4" t="str">
+        <x:v>大型上市移动发行商；2025年收入约KRW 2.7万亿级，旗下含 Kabam/SpinX/Jam City 等资产。</x:v>
+      </x:c>
+      <x:c r="F9" s="4" t="str">
+        <x:v>MARVEL Future Fight、Seven Knights、Solo Leveling: ARISE、Ni no Kuni: Cross Worlds。</x:v>
+      </x:c>
+      <x:c r="G9" s="4" t="str">
+        <x:v>netmarblebiz@netmarble.com</x:v>
+      </x:c>
+      <x:c r="H9" s="4" t="str">
+        <x:v>官网公开 business 邮箱。</x:v>
+      </x:c>
+      <x:c r="I9" s="4" t="str">
         <x:v>2025 results page describes Netmarble as leading developer/publisher and lists major subsidiaries/holdings.</x:v>
       </x:c>
-      <x:c r="F9" s="4" t="str">
+      <x:c r="J9" s="4" t="str">
         <x:v>Publishing; MG; strategic investment; acquisition if scale proven</x:v>
       </x:c>
-      <x:c r="G9" s="4" t="str">
+      <x:c r="K9" s="4" t="str">
         <x:v>Global Publishing; Corporate Development; Investment</x:v>
       </x:c>
-      <x:c r="H9" s="4" t="str">
+      <x:c r="L9" s="4" t="str">
         <x:v>https://company.netmarble.com/en</x:v>
       </x:c>
-      <x:c r="I9" s="4" t="str">
+      <x:c r="M9" s="4" t="str">
         <x:v>Pitch as a validated US-tested mobile F2P title adjacent to their global mobile portfolio.</x:v>
       </x:c>
-      <x:c r="J9" s="4" t="str">
+      <x:c r="N9" s="4" t="str">
         <x:v>Korean buyers may ask for UA/raw cohort data quickly; prepare CPI, D1/D7/D30, payback and creative tests.</x:v>
       </x:c>
-      <x:c r="K9" s="4" t="str">
+      <x:c r="O9" s="4" t="str">
         <x:v>https://ch.netmarble.com/Eng/Newsroom/Detail?bbs_code=1020&amp;post_seq=6475&amp;post_tag=NETMARBLE | https://company.netmarble.com/en/company/about | https://company.netmarble.com/en/ir</x:v>
       </x:c>
     </x:row>
@@ -8621,24 +9717,36 @@
         <x:v>78</x:v>
       </x:c>
       <x:c r="E10" s="4" t="str">
+        <x:v>上市游戏/投资集团；年收入数百亿日元级，WFS/GREE Studios/Pokelabo 等子品牌。</x:v>
+      </x:c>
+      <x:c r="F10" s="4" t="str">
+        <x:v>Heaven Burns Red、Another Eden、Fishing Star、Magia Exedra/Pokelabo 相关项目。</x:v>
+      </x:c>
+      <x:c r="G10" s="4" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="H10" s="4" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://www.wfs.games/en/contact/</x:v>
+      </x:c>
+      <x:c r="I10" s="4" t="str">
         <x:v>GREE business overview lists Game and Investment businesses; 2025 restructuring moved live service games into WFS.</x:v>
       </x:c>
-      <x:c r="F10" s="4" t="str">
+      <x:c r="J10" s="4" t="str">
         <x:v>Publishing; strategic investment; Japan/Asia partnership</x:v>
       </x:c>
-      <x:c r="G10" s="4" t="str">
+      <x:c r="K10" s="4" t="str">
         <x:v>WFS live-service; GREE investment; business development</x:v>
       </x:c>
-      <x:c r="H10" s="4" t="str">
+      <x:c r="L10" s="4" t="str">
         <x:v>https://www.wfs.games/en/contact/</x:v>
       </x:c>
-      <x:c r="I10" s="4" t="str">
+      <x:c r="M10" s="4" t="str">
         <x:v>Present as a mobile live-service title with proven Western acquisition metrics and expandable content cadence.</x:v>
       </x:c>
-      <x:c r="J10" s="4" t="str">
+      <x:c r="N10" s="4" t="str">
         <x:v>Japanese buyers may prefer stronger localization/IP plan; use concise Japanese follow-up after English opener.</x:v>
       </x:c>
-      <x:c r="K10" s="4" t="str">
+      <x:c r="O10" s="4" t="str">
         <x:v>https://gree.co.jp/jp/en/business/index.html | https://www.wfs.games/en/ | https://www.gematsu.com/2024/11/gree-establishes-gree-studios-to-manage-consumer-games-business-live-service-games-business-absorbed-by-wfs</x:v>
       </x:c>
     </x:row>
@@ -8656,24 +9764,36 @@
         <x:v>76</x:v>
       </x:c>
       <x:c r="E11" s="4" t="str">
+        <x:v>上市数字娱乐集团；年收入千亿日元级，Monster Strike 为核心现金流。</x:v>
+      </x:c>
+      <x:c r="F11" s="4" t="str">
+        <x:v>Monster Strike、Kotodaman、TIPSTAR/数字娱乐业务。</x:v>
+      </x:c>
+      <x:c r="G11" s="4" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="H11" s="4" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://invest.mixi.co.jp/</x:v>
+      </x:c>
+      <x:c r="I11" s="4" t="str">
         <x:v>MIXI corporate profile lists Digital Entertainment and Investment; investment site shows active investing activity.</x:v>
       </x:c>
-      <x:c r="F11" s="4" t="str">
+      <x:c r="J11" s="4" t="str">
         <x:v>Strategic investment; publishing; Japan co-operation; MG</x:v>
       </x:c>
-      <x:c r="G11" s="4" t="str">
+      <x:c r="K11" s="4" t="str">
         <x:v>Digital Entertainment; Investment</x:v>
       </x:c>
-      <x:c r="H11" s="4" t="str">
+      <x:c r="L11" s="4" t="str">
         <x:v>https://invest.mixi.co.jp/</x:v>
       </x:c>
-      <x:c r="I11" s="4" t="str">
+      <x:c r="M11" s="4" t="str">
         <x:v>Pitch as a mobile F2P title with US proof, asking whether investment or publishing support fits their digital entertainment goals.</x:v>
       </x:c>
-      <x:c r="J11" s="4" t="str">
+      <x:c r="N11" s="4" t="str">
         <x:v>Japanese buyers may prefer stronger localization/IP plan; use concise Japanese follow-up after English opener.</x:v>
       </x:c>
-      <x:c r="K11" s="4" t="str">
+      <x:c r="O11" s="4" t="str">
         <x:v>https://mixi.co.jp/en/company/profile/ | https://mixi.co.jp/en/business/investment/ | https://invest.mixi.co.jp/</x:v>
       </x:c>
     </x:row>
@@ -8691,24 +9811,36 @@
         <x:v>76</x:v>
       </x:c>
       <x:c r="E12" s="4" t="str">
+        <x:v>Smilegate 集团发行板块；集团级公司，全球员工/业务规模千人级。</x:v>
+      </x:c>
+      <x:c r="F12" s="4" t="str">
+        <x:v>Epic Seven、Lost Ark 全球业务、Smilegate Megaport 发行体系。</x:v>
+      </x:c>
+      <x:c r="G12" s="4" t="str">
+        <x:v>sgp_biz@smilegate.com</x:v>
+      </x:c>
+      <x:c r="H12" s="4" t="str">
+        <x:v>Smilegate Megaport 业务页公开邮箱。</x:v>
+      </x:c>
+      <x:c r="I12" s="4" t="str">
         <x:v>Smilegate official site highlights publishing activity and global business expansion.</x:v>
       </x:c>
-      <x:c r="F12" s="4" t="str">
+      <x:c r="J12" s="4" t="str">
         <x:v>Publishing; MG; strategic partnership; minority investment</x:v>
       </x:c>
-      <x:c r="G12" s="4" t="str">
+      <x:c r="K12" s="4" t="str">
         <x:v>Smilegate Megaport; Global Business; Investment</x:v>
       </x:c>
-      <x:c r="H12" s="4" t="str">
+      <x:c r="L12" s="4" t="str">
         <x:v>https://www.smilegate.com/en/</x:v>
       </x:c>
-      <x:c r="I12" s="4" t="str">
+      <x:c r="M12" s="4" t="str">
         <x:v>Lead with global-ready mobile F2P and ask whether Megaport wants a US-tested casual simulation title.</x:v>
       </x:c>
-      <x:c r="J12" s="4" t="str">
+      <x:c r="N12" s="4" t="str">
         <x:v>Korean buyers may ask for UA/raw cohort data quickly; prepare CPI, D1/D7/D30, payback and creative tests.</x:v>
       </x:c>
-      <x:c r="K12" s="4" t="str">
+      <x:c r="O12" s="4" t="str">
         <x:v>https://www.smilegate.com/en/ | https://www.smilegate.com/business/megaport.do | https://www.smilegate.com/en/news/list.do</x:v>
       </x:c>
     </x:row>
@@ -8726,24 +9858,36 @@
         <x:v>72</x:v>
       </x:c>
       <x:c r="E13" s="4" t="str">
+        <x:v>上市移动游戏公司；资本金约89.3亿日元，移动游戏开发运营团队。</x:v>
+      </x:c>
+      <x:c r="F13" s="4" t="str">
+        <x:v>Bleach: Brave Souls、Captain Tsubasa: Dream Team、Love Live! 相关历史项目。</x:v>
+      </x:c>
+      <x:c r="G13" s="4" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="H13" s="4" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://www.klab.com/en/contact/</x:v>
+      </x:c>
+      <x:c r="I13" s="4" t="str">
         <x:v>KLab official releases describe global mobile launches and overseas support model.</x:v>
       </x:c>
-      <x:c r="F13" s="4" t="str">
+      <x:c r="J13" s="4" t="str">
         <x:v>Publishing; co-development; Japan/IP collaboration; MG</x:v>
       </x:c>
-      <x:c r="G13" s="4" t="str">
+      <x:c r="K13" s="4" t="str">
         <x:v>Overseas Game Development Support; Business Development</x:v>
       </x:c>
-      <x:c r="H13" s="4" t="str">
+      <x:c r="L13" s="4" t="str">
         <x:v>https://www.klab.com/en/contact/</x:v>
       </x:c>
-      <x:c r="I13" s="4" t="str">
+      <x:c r="M13" s="4" t="str">
         <x:v>Emphasize that the game does not require major Japanese IP, but can leverage KLab's global mobile operating experience.</x:v>
       </x:c>
-      <x:c r="J13" s="4" t="str">
+      <x:c r="N13" s="4" t="str">
         <x:v>Japanese buyers may prefer stronger localization/IP plan; use concise Japanese follow-up after English opener.</x:v>
       </x:c>
-      <x:c r="K13" s="4" t="str">
+      <x:c r="O13" s="4" t="str">
         <x:v>https://www.klab.com/en/ | https://www.klab.com/en/press/release/2025/0801/flyhigh.html | https://www.klab.com/en/ir/</x:v>
       </x:c>
     </x:row>
@@ -8761,24 +9905,36 @@
         <x:v>72</x:v>
       </x:c>
       <x:c r="E14" s="4" t="str">
+        <x:v>上市游戏发行商；年收入数千亿韩元级，拥有 XLGAMES/Lionheart/Ocean Drive 等工作室。</x:v>
+      </x:c>
+      <x:c r="F14" s="4" t="str">
+        <x:v>Odin: Valhalla Rising、Uma Musume KR、Eversoul、ArcheAge War。</x:v>
+      </x:c>
+      <x:c r="G14" s="4" t="str">
+        <x:v>contact@kakaogames.com</x:v>
+      </x:c>
+      <x:c r="H14" s="4" t="str">
+        <x:v>官网 Contact 页面公开邮箱；页面标注 receive-only，建议并行表单/LinkedIn。</x:v>
+      </x:c>
+      <x:c r="I14" s="4" t="str">
         <x:v>Official site positions Kakao Games as global multi-platform publisher with mobile portfolio and IR materials.</x:v>
       </x:c>
-      <x:c r="F14" s="4" t="str">
+      <x:c r="J14" s="4" t="str">
         <x:v>Publishing; MG; strategic investment; Korea/Japan operation</x:v>
       </x:c>
-      <x:c r="G14" s="4" t="str">
+      <x:c r="K14" s="4" t="str">
         <x:v>Global Business; Mobile Publishing; Investment</x:v>
       </x:c>
-      <x:c r="H14" s="4" t="str">
+      <x:c r="L14" s="4" t="str">
         <x:v>https://www.kakaogamescorp.com/en/customer/contact</x:v>
       </x:c>
-      <x:c r="I14" s="4" t="str">
+      <x:c r="M14" s="4" t="str">
         <x:v>Pitch as a mobile F2P project with US proof and a clear Japan/Korea localization path.</x:v>
       </x:c>
-      <x:c r="J14" s="4" t="str">
+      <x:c r="N14" s="4" t="str">
         <x:v>Korean buyers may ask for UA/raw cohort data quickly; prepare CPI, D1/D7/D30, payback and creative tests.</x:v>
       </x:c>
-      <x:c r="K14" s="4" t="str">
+      <x:c r="O14" s="4" t="str">
         <x:v>https://www.kakaogamescorp.com/en | https://www.kakaogamescorp.com/en/ir/irData | https://www.kakaogamescorp.com/en/game</x:v>
       </x:c>
     </x:row>
@@ -8796,24 +9952,36 @@
         <x:v>72</x:v>
       </x:c>
       <x:c r="E15" s="4" t="str">
+        <x:v>上市发行/开发公司；年收入数千亿韩元级，PC/主机/移动组合。</x:v>
+      </x:c>
+      <x:c r="F15" s="4" t="str">
+        <x:v>Lies of P、BrownDust2、Sanabi、DJMAX RESPECT。</x:v>
+      </x:c>
+      <x:c r="G15" s="4" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="H15" s="4" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://www.neowiz.com/neowiz</x:v>
+      </x:c>
+      <x:c r="I15" s="4" t="str">
         <x:v>Recent investor/news coverage shows focus on global IP and partner collaborations; official IR has in-house/publishing pipeline.</x:v>
       </x:c>
-      <x:c r="F15" s="4" t="str">
+      <x:c r="J15" s="4" t="str">
         <x:v>Publishing; co-development; strategic investment</x:v>
       </x:c>
-      <x:c r="G15" s="4" t="str">
+      <x:c r="K15" s="4" t="str">
         <x:v>Global Publishing; Business Development; Corporate Strategy</x:v>
       </x:c>
-      <x:c r="H15" s="4" t="str">
+      <x:c r="L15" s="4" t="str">
         <x:v>https://www.neowiz.com/neowiz</x:v>
       </x:c>
-      <x:c r="I15" s="4" t="str">
+      <x:c r="M15" s="4" t="str">
         <x:v>Position as external global IP candidate, with mobile casual economics distinct from their PC/console pipeline.</x:v>
       </x:c>
-      <x:c r="J15" s="4" t="str">
+      <x:c r="N15" s="4" t="str">
         <x:v>Korean buyers may ask for UA/raw cohort data quickly; prepare CPI, D1/D7/D30, payback and creative tests.</x:v>
       </x:c>
-      <x:c r="K15" s="4" t="str">
+      <x:c r="O15" s="4" t="str">
         <x:v>https://cdn.neowiz.com/neowiz-site/assets/ir-library/Q1-2025_NWZ_PPT_EN-dggcl9vz-xkoamocn.pdf | https://www.neowiz.com/neowiz | https://store.steampowered.com/publisher/NEOWIZ</x:v>
       </x:c>
     </x:row>
@@ -8831,24 +9999,36 @@
         <x:v>69</x:v>
       </x:c>
       <x:c r="E16" s="4" t="str">
+        <x:v>上市移动游戏公司；年收入数百亿日元级，另有 COLOPL NEXT 投资平台。</x:v>
+      </x:c>
+      <x:c r="F16" s="4" t="str">
+        <x:v>White Cat Project、Dragon Project、Alice Gear Aegis；COLOPL NEXT 投资。</x:v>
+      </x:c>
+      <x:c r="G16" s="4" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="H16" s="4" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://www.coloplnext.co.jp/en/</x:v>
+      </x:c>
+      <x:c r="I16" s="4" t="str">
         <x:v>COLOPL official pages cover mobile entertainment; COLOPL NEXT provides venture investment pathway.</x:v>
       </x:c>
-      <x:c r="F16" s="4" t="str">
+      <x:c r="J16" s="4" t="str">
         <x:v>Strategic investment; publishing; co-development</x:v>
       </x:c>
-      <x:c r="G16" s="4" t="str">
+      <x:c r="K16" s="4" t="str">
         <x:v>COLOPL NEXT; Game Business; BD</x:v>
       </x:c>
-      <x:c r="H16" s="4" t="str">
+      <x:c r="L16" s="4" t="str">
         <x:v>https://www.coloplnext.co.jp/en/</x:v>
       </x:c>
-      <x:c r="I16" s="4" t="str">
+      <x:c r="M16" s="4" t="str">
         <x:v>Pitch as a mobile casual-adventure studio with US proof and potential portfolio extension.</x:v>
       </x:c>
-      <x:c r="J16" s="4" t="str">
+      <x:c r="N16" s="4" t="str">
         <x:v>Japanese buyers may prefer stronger localization/IP plan; use concise Japanese follow-up after English opener.</x:v>
       </x:c>
-      <x:c r="K16" s="4" t="str">
+      <x:c r="O16" s="4" t="str">
         <x:v>https://colopl.co.jp/en/ | https://www.coloplnext.co.jp/en/ | https://colopl.co.jp/en/ir/</x:v>
       </x:c>
     </x:row>
@@ -8866,24 +10046,36 @@
         <x:v>69</x:v>
       </x:c>
       <x:c r="E17" s="4" t="str">
+        <x:v>上市移动游戏/区块链娱乐公司；年收入百亿日元级。</x:v>
+      </x:c>
+      <x:c r="F17" s="4" t="str">
+        <x:v>Brave Frontier、Final Fantasy Brave Exvius、Aster Tatariqus。</x:v>
+      </x:c>
+      <x:c r="G17" s="4" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="H17" s="4" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://gu3.co.jp/en/contact/</x:v>
+      </x:c>
+      <x:c r="I17" s="4" t="str">
         <x:v>gumi official pages describe mobile online game experience and investment/business cooperation in emerging entertainment.</x:v>
       </x:c>
-      <x:c r="F17" s="4" t="str">
+      <x:c r="J17" s="4" t="str">
         <x:v>Publishing; co-development; strategic investment; asset deal</x:v>
       </x:c>
-      <x:c r="G17" s="4" t="str">
+      <x:c r="K17" s="4" t="str">
         <x:v>Game business; Investment/Blockchain strategy; BD</x:v>
       </x:c>
-      <x:c r="H17" s="4" t="str">
+      <x:c r="L17" s="4" t="str">
         <x:v>https://gu3.co.jp/en/contact/</x:v>
       </x:c>
-      <x:c r="I17" s="4" t="str">
+      <x:c r="M17" s="4" t="str">
         <x:v>Position as a proven F2P mobile project with less speculative risk than early blockchain content.</x:v>
       </x:c>
-      <x:c r="J17" s="4" t="str">
+      <x:c r="N17" s="4" t="str">
         <x:v>Japanese buyers may prefer stronger localization/IP plan; use concise Japanese follow-up after English opener.</x:v>
       </x:c>
-      <x:c r="K17" s="4" t="str">
+      <x:c r="O17" s="4" t="str">
         <x:v>https://gu3.co.jp/en/ | https://gu3.co.jp/en/blockchain/ | https://gu3.co.jp/en/ir/</x:v>
       </x:c>
     </x:row>
@@ -8901,24 +10093,36 @@
         <x:v>69</x:v>
       </x:c>
       <x:c r="E18" s="4" t="str">
+        <x:v>上市移动/在线游戏公司；年收入千亿日元级，Puzzle &amp; Dragons 为核心。</x:v>
+      </x:c>
+      <x:c r="F18" s="4" t="str">
+        <x:v>Puzzle &amp; Dragons、Ragnarok Online DS/相关合作、Ninjala。</x:v>
+      </x:c>
+      <x:c r="G18" s="4" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="H18" s="4" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://www.gungho.co.jp/en/contact/</x:v>
+      </x:c>
+      <x:c r="I18" s="4" t="str">
         <x:v>Official corporate pages show mobile game operations, global group, and investor communications.</x:v>
       </x:c>
-      <x:c r="F18" s="4" t="str">
+      <x:c r="J18" s="4" t="str">
         <x:v>Publishing; MG; co-development; minority investment</x:v>
       </x:c>
-      <x:c r="G18" s="4" t="str">
+      <x:c r="K18" s="4" t="str">
         <x:v>Business Development; Global Publishing</x:v>
       </x:c>
-      <x:c r="H18" s="4" t="str">
+      <x:c r="L18" s="4" t="str">
         <x:v>https://www.gungho.co.jp/en/contact/</x:v>
       </x:c>
-      <x:c r="I18" s="4" t="str">
+      <x:c r="M18" s="4" t="str">
         <x:v>Frame as a casual F2P simulation project with proven retention and low creative risk.</x:v>
       </x:c>
-      <x:c r="J18" s="4" t="str">
+      <x:c r="N18" s="4" t="str">
         <x:v>Japanese buyers may prefer stronger localization/IP plan; use concise Japanese follow-up after English opener.</x:v>
       </x:c>
-      <x:c r="K18" s="4" t="str">
+      <x:c r="O18" s="4" t="str">
         <x:v>https://www.gungho.co.jp/en/ | https://www.gungho.co.jp/en/ir/ | https://www.gungho.co.jp/en/game/</x:v>
       </x:c>
     </x:row>
@@ -8936,24 +10140,36 @@
         <x:v>69</x:v>
       </x:c>
       <x:c r="E19" s="4" t="str">
+        <x:v>中小型休闲手游公司；公开公司资料常见规模约51-200人级。</x:v>
+      </x:c>
+      <x:c r="F19" s="4" t="str">
+        <x:v>Burger Please!、Outlets Rush、Pizza Ready! 等混合休闲发行案例。</x:v>
+      </x:c>
+      <x:c r="G19" s="4" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="H19" s="4" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://supercent.io/</x:v>
+      </x:c>
+      <x:c r="I19" s="4" t="str">
         <x:v>Official site positions Supercent around casual mobile publishing and developer partnerships.</x:v>
       </x:c>
-      <x:c r="F19" s="4" t="str">
+      <x:c r="J19" s="4" t="str">
         <x:v>Publishing; MG; UA partnership; lightweight investment</x:v>
       </x:c>
-      <x:c r="G19" s="4" t="str">
+      <x:c r="K19" s="4" t="str">
         <x:v>Publishing; Developer Relations</x:v>
       </x:c>
-      <x:c r="H19" s="4" t="str">
+      <x:c r="L19" s="4" t="str">
         <x:v>https://supercent.io/</x:v>
       </x:c>
-      <x:c r="I19" s="4" t="str">
+      <x:c r="M19" s="4" t="str">
         <x:v>Lead with CPI/retention details and ask for hybrid-casual scaling perspective.</x:v>
       </x:c>
-      <x:c r="J19" s="4" t="str">
+      <x:c r="N19" s="4" t="str">
         <x:v>Korean buyers may ask for UA/raw cohort data quickly; prepare CPI, D1/D7/D30, payback and creative tests.</x:v>
       </x:c>
-      <x:c r="K19" s="4" t="str">
+      <x:c r="O19" s="4" t="str">
         <x:v>https://supercent.io/ | https://www.linkedin.com/company/supercent/ | https://supercent.io/contact</x:v>
       </x:c>
     </x:row>
@@ -8971,24 +10187,36 @@
         <x:v>67</x:v>
       </x:c>
       <x:c r="E20" s="4" t="str">
+        <x:v>中小型休闲手游公司；公开公司资料常见规模约51-200人级。</x:v>
+      </x:c>
+      <x:c r="F20" s="4" t="str">
+        <x:v>Random Dice 系列、B.B.TAN、Wild Tamer；Supercent 生态相关。</x:v>
+      </x:c>
+      <x:c r="G20" s="4" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="H20" s="4" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://111percent.net/en/contact/</x:v>
+      </x:c>
+      <x:c r="I20" s="4" t="str">
         <x:v>Official site lists mobile casual portfolio and company focus.</x:v>
       </x:c>
-      <x:c r="F20" s="4" t="str">
+      <x:c r="J20" s="4" t="str">
         <x:v>Publishing; UA partnership; strategic collaboration</x:v>
       </x:c>
-      <x:c r="G20" s="4" t="str">
+      <x:c r="K20" s="4" t="str">
         <x:v>Publishing; Business Development; Supercent relationship</x:v>
       </x:c>
-      <x:c r="H20" s="4" t="str">
+      <x:c r="L20" s="4" t="str">
         <x:v>https://111percent.net/en/contact/</x:v>
       </x:c>
-      <x:c r="I20" s="4" t="str">
+      <x:c r="M20" s="4" t="str">
         <x:v>Position as proven casual-sim title; ask whether 111% or Supercent is the right evaluation path.</x:v>
       </x:c>
-      <x:c r="J20" s="4" t="str">
+      <x:c r="N20" s="4" t="str">
         <x:v>Korean buyers may ask for UA/raw cohort data quickly; prepare CPI, D1/D7/D30, payback and creative tests.</x:v>
       </x:c>
-      <x:c r="K20" s="4" t="str">
+      <x:c r="O20" s="4" t="str">
         <x:v>https://111percent.net/en/ | https://111percent.net/en/games/ | https://www.linkedin.com/company/111percent/</x:v>
       </x:c>
     </x:row>
@@ -9006,31 +10234,43 @@
         <x:v>66</x:v>
       </x:c>
       <x:c r="E21" s="4" t="str">
+        <x:v>大型上市媒体/IP集团；集团年收入数千亿日元级，游戏为内容/IP组合之一。</x:v>
+      </x:c>
+      <x:c r="F21" s="4" t="str">
+        <x:v>FromSoftware/Spike Chunsoft 相关持股与出版/IP生态；游戏/IP投资合作。</x:v>
+      </x:c>
+      <x:c r="G21" s="4" t="str">
+        <x:v>未公开商务邮箱</x:v>
+      </x:c>
+      <x:c r="H21" s="4" t="str">
+        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://group.kadokawa.co.jp/global/contact/</x:v>
+      </x:c>
+      <x:c r="I21" s="4" t="str">
         <x:v>KADOKAWA integrated reports discuss game developer investments and IP/global expansion.</x:v>
       </x:c>
-      <x:c r="F21" s="4" t="str">
+      <x:c r="J21" s="4" t="str">
         <x:v>Strategic investment; IP/game partnership; acquisition if IP angle strong</x:v>
       </x:c>
-      <x:c r="G21" s="4" t="str">
+      <x:c r="K21" s="4" t="str">
         <x:v>Game business; Corporate Strategy; Investment/Alliance</x:v>
       </x:c>
-      <x:c r="H21" s="4" t="str">
+      <x:c r="L21" s="4" t="str">
         <x:v>https://group.kadokawa.co.jp/global/contact/</x:v>
       </x:c>
-      <x:c r="I21" s="4" t="str">
+      <x:c r="M21" s="4" t="str">
         <x:v>Best if pitched as an original world/IP plus mobile live-service system, not just a pure UA play.</x:v>
       </x:c>
-      <x:c r="J21" s="4" t="str">
+      <x:c r="N21" s="4" t="str">
         <x:v>Japanese buyers may prefer stronger localization/IP plan; use concise Japanese follow-up after English opener.</x:v>
       </x:c>
-      <x:c r="K21" s="4" t="str">
+      <x:c r="O21" s="4" t="str">
         <x:v>https://group.kadokawa.co.jp/global/ | https://group.kadokawa.co.jp/ir/library/integrated_report.html | https://group.kadokawa.co.jp/media/ir/media-download/1851/8394a61e1784306e/</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re8a20f075be64a50"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc5a6857adb054212"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10084,7 +11324,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R91ae4434286e486d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf23139fba65f4ca3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10279,7 +11519,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2621b4c9bbab445e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff5bf7e430864123"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13671,7 +14911,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R48e9539524394eef"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R691547030d4e4681"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add rihanfx email search strategy
</commit_message>
<xml_diff>
--- a/contact/rihanfx/jp_kr_game_outreach_workbook.xlsx
+++ b/contact/rihanfx/jp_kr_game_outreach_workbook.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README_Summary" sheetId="1" r:id="R0b755d684cfa4e50"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Longlist_80" sheetId="2" r:id="R2e6ad334a0ea4c97"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top20_Playbook" sheetId="3" r:id="R66f3563152ad45c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoring_Model" sheetId="4" r:id="R83937186cec64efe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outreach_Pipeline" sheetId="5" r:id="R12b897121f1c4112"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Templates" sheetId="6" r:id="Rf11a50eff84b4ce1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source_Registry" sheetId="7" r:id="R682a5bf3cd7a4209"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README_Summary" sheetId="1" r:id="R71919adb39284898"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Longlist_80" sheetId="2" r:id="Rbfc0e2794e6e4ddd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top20_Playbook" sheetId="3" r:id="R420cb273b0f04fe9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoring_Model" sheetId="4" r:id="Rb18f98d9e4b348d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outreach_Pipeline" sheetId="5" r:id="R0957451879c24738"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Templates" sheetId="6" r:id="R1ab3165cbdbd4464"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source_Registry" sheetId="7" r:id="Rabcb9e6bb63b447d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2709,13 +2709,13 @@
         <x:v>中小型休闲手游公司；公开公司资料常见规模约51-200人级。</x:v>
       </x:c>
       <x:c r="AG19" s="7" t="str">
-        <x:v>Burger Please!、Outlets Rush、Pizza Ready! 等混合休闲发行案例。</x:v>
+        <x:v>Burger Please!、Outlets Rush、Pizza Ready!、Snake Clash；官网显示累计下载 1.5B+、累计收入 $380M+。</x:v>
       </x:c>
       <x:c r="AH19" s="7" t="str">
-        <x:v>未公开商务邮箱</x:v>
+        <x:v>help@supercent.io</x:v>
       </x:c>
       <x:c r="AI19" s="7" t="str">
-        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://supercent.io/</x:v>
+        <x:v>官网英文 About、韩文公司页、Terms/Privacy 等页面均公开 help@supercent.io；偏通用/客服邮箱，BD仍建议并行 Submit Your Game/Publishing 入口。</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -9254,7 +9254,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R85b88eca23694c7b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R266f4ee786d14b80"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10143,13 +10143,13 @@
         <x:v>中小型休闲手游公司；公开公司资料常见规模约51-200人级。</x:v>
       </x:c>
       <x:c r="F19" s="4" t="str">
-        <x:v>Burger Please!、Outlets Rush、Pizza Ready! 等混合休闲发行案例。</x:v>
+        <x:v>Burger Please!、Outlets Rush、Pizza Ready!、Snake Clash；官网显示累计下载 1.5B+、累计收入 $380M+。</x:v>
       </x:c>
       <x:c r="G19" s="4" t="str">
-        <x:v>未公开商务邮箱</x:v>
+        <x:v>help@supercent.io</x:v>
       </x:c>
       <x:c r="H19" s="4" t="str">
-        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://supercent.io/</x:v>
+        <x:v>官网英文 About、韩文公司页、Terms/Privacy 等页面均公开 help@supercent.io；偏通用/客服邮箱，BD仍建议并行 Submit Your Game/Publishing 入口。</x:v>
       </x:c>
       <x:c r="I19" s="4" t="str">
         <x:v>Official site positions Supercent around casual mobile publishing and developer partnerships.</x:v>
@@ -10270,7 +10270,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc5a6857adb054212"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R17c09e927ac14f12"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11324,7 +11324,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf23139fba65f4ca3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a42aeb4f7fa49a3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11519,7 +11519,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff5bf7e430864123"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0abf06b158554755"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14911,7 +14911,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R691547030d4e4681"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R56e55f6e73a94b50"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Improve rihanfx email coverage
</commit_message>
<xml_diff>
--- a/contact/rihanfx/jp_kr_game_outreach_workbook.xlsx
+++ b/contact/rihanfx/jp_kr_game_outreach_workbook.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README_Summary" sheetId="1" r:id="R71919adb39284898"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Longlist_80" sheetId="2" r:id="Rbfc0e2794e6e4ddd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top20_Playbook" sheetId="3" r:id="R420cb273b0f04fe9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoring_Model" sheetId="4" r:id="Rb18f98d9e4b348d0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outreach_Pipeline" sheetId="5" r:id="R0957451879c24738"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Templates" sheetId="6" r:id="R1ab3165cbdbd4464"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source_Registry" sheetId="7" r:id="Rabcb9e6bb63b447d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README_Summary" sheetId="1" r:id="Rf9a7b6f584844f8c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Longlist_80" sheetId="2" r:id="Rbfb1ddcc39f348d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top20_Playbook" sheetId="3" r:id="R84de2f567e2d4678"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoring_Model" sheetId="4" r:id="R5aed2853f0d14c70"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outreach_Pipeline" sheetId="5" r:id="R3b55977dd4d64d31"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Templates" sheetId="6" r:id="R2f03064fce614fe7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source_Registry" sheetId="7" r:id="Refdc45e2e79847cd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2397,10 +2397,10 @@
         <x:v>White Cat Project、Dragon Project、Alice Gear Aegis；COLOPL NEXT 投资。</x:v>
       </x:c>
       <x:c r="AH16" s="7" t="str">
-        <x:v>未公开商务邮箱</x:v>
+        <x:v>help@colopl.jp</x:v>
       </x:c>
       <x:c r="AI16" s="7" t="str">
-        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://www.coloplnext.co.jp/en/</x:v>
+        <x:v>官网 Contact 页面公开 help@；偏客服/通用邮箱，另有多款游戏 support 邮箱已排除；BD仍建议并行 COLOPL NEXT/官网入口。</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -4497,10 +4497,10 @@
         <x:v>BanG Dream!, D4DJ, card games, mobile games</x:v>
       </x:c>
       <x:c r="AH36" s="7" t="str">
-        <x:v>未公开商务邮箱</x:v>
+        <x:v>ir@bushiroad.com; support@bushiroad.com</x:v>
       </x:c>
       <x:c r="AI36" s="7" t="str">
-        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://bushiroad.co.jp/en/contact/</x:v>
+        <x:v>英文 Contact 页面公开 IR/support 邮箱；非发行BD专属，建议邮件请求转给游戏业务/投资合作负责人。</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
@@ -5862,10 +5862,10 @@
         <x:v>Exos Heroes, Undecember, Buried Stars; mobile/PC publishing</x:v>
       </x:c>
       <x:c r="AH49" s="7" t="str">
-        <x:v>未公开商务邮箱</x:v>
+        <x:v>linegames_biz@line.games; ir@line.games</x:v>
       </x:c>
       <x:c r="AI49" s="7" t="str">
-        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://line.games/en/contact</x:v>
+        <x:v>官网 Company 页面公开 biz/IR 邮箱；BD优先 linegames_biz@，game_service support 邮箱已排除。</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
@@ -7332,10 +7332,10 @@
         <x:v>Gran Saga; Chrono Odyssey; mobile/PC/console ambitions</x:v>
       </x:c>
       <x:c r="AH63" s="7" t="str">
-        <x:v>未公开商务邮箱</x:v>
+        <x:v>business@npixel.co.kr</x:v>
       </x:c>
       <x:c r="AI63" s="7" t="str">
-        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://npixel.co.kr/en/contact</x:v>
+        <x:v>官网根页面公开 business 邮箱；同页 npixel@/privacy@/recruit@ 未作为BD首选。</x:v>
       </x:c>
     </x:row>
     <x:row r="64">
@@ -7437,10 +7437,10 @@
         <x:v>Ikemen Series; mobile entertainment and IP content</x:v>
       </x:c>
       <x:c r="AH64" s="7" t="str">
-        <x:v>未公开商务邮箱</x:v>
+        <x:v>otoiawase@cybird.co.jp</x:v>
       </x:c>
       <x:c r="AI64" s="7" t="str">
-        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://www.cybird.co.jp/en/contact/</x:v>
+        <x:v>官网 Contact 页面公开日文 inquiry 邮箱；适合作为日本本地化/商务转接入口。</x:v>
       </x:c>
     </x:row>
     <x:row r="65">
@@ -8382,10 +8382,10 @@
         <x:v>Blade, Boxing Star, mobile action/social titles</x:v>
       </x:c>
       <x:c r="AH73" s="7" t="str">
-        <x:v>未公开商务邮箱</x:v>
+        <x:v>business@433.co.kr; ftt_bd@433.co.kr</x:v>
       </x:c>
       <x:c r="AI73" s="7" t="str">
-        <x:v>未找到公开商务邮箱；建议使用官方联系入口：http://www.433.co.kr/</x:v>
+        <x:v>官网 Contact 页面公开 business 与 BD 邮箱；BD优先 business@，ftt_bd@ 可并行。</x:v>
       </x:c>
     </x:row>
     <x:row r="74">
@@ -9254,7 +9254,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R266f4ee786d14b80"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1148c88ff1f44400"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10005,10 +10005,10 @@
         <x:v>White Cat Project、Dragon Project、Alice Gear Aegis；COLOPL NEXT 投资。</x:v>
       </x:c>
       <x:c r="G16" s="4" t="str">
-        <x:v>未公开商务邮箱</x:v>
+        <x:v>help@colopl.jp</x:v>
       </x:c>
       <x:c r="H16" s="4" t="str">
-        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://www.coloplnext.co.jp/en/</x:v>
+        <x:v>官网 Contact 页面公开 help@；偏客服/通用邮箱，另有多款游戏 support 邮箱已排除；BD仍建议并行 COLOPL NEXT/官网入口。</x:v>
       </x:c>
       <x:c r="I16" s="4" t="str">
         <x:v>COLOPL official pages cover mobile entertainment; COLOPL NEXT provides venture investment pathway.</x:v>
@@ -10270,7 +10270,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R17c09e927ac14f12"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0613d74db6cd4b6f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11324,7 +11324,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a42aeb4f7fa49a3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb36f010631d49c4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11519,7 +11519,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0abf06b158554755"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71f018ae6f9b4526"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14911,7 +14911,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R56e55f6e73a94b50"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf1d4ff15ff764e34"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add 111Percent email discovery
</commit_message>
<xml_diff>
--- a/contact/rihanfx/jp_kr_game_outreach_workbook.xlsx
+++ b/contact/rihanfx/jp_kr_game_outreach_workbook.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README_Summary" sheetId="1" r:id="Rf9a7b6f584844f8c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Longlist_80" sheetId="2" r:id="Rbfb1ddcc39f348d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top20_Playbook" sheetId="3" r:id="R84de2f567e2d4678"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoring_Model" sheetId="4" r:id="R5aed2853f0d14c70"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outreach_Pipeline" sheetId="5" r:id="R3b55977dd4d64d31"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Templates" sheetId="6" r:id="R2f03064fce614fe7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source_Registry" sheetId="7" r:id="Refdc45e2e79847cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README_Summary" sheetId="1" r:id="R09dda58d969448ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Longlist_80" sheetId="2" r:id="R57335e9ab5664944"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top20_Playbook" sheetId="3" r:id="R89268a58c97d4a01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoring_Model" sheetId="4" r:id="Rf27884b0fb914144"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outreach_Pipeline" sheetId="5" r:id="R0743e28e701b44d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Templates" sheetId="6" r:id="R67fa21db76b04499"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source_Registry" sheetId="7" r:id="Rd147b87409494327"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2817,10 +2817,10 @@
         <x:v>Random Dice 系列、B.B.TAN、Wild Tamer；Supercent 生态相关。</x:v>
       </x:c>
       <x:c r="AH20" s="7" t="str">
-        <x:v>未公开商务邮箱</x:v>
+        <x:v>business@111percent.net; branding@111percent.net; marketing@111percent.net</x:v>
       </x:c>
       <x:c r="AI20" s="7" t="str">
-        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://111percent.net/en/contact/</x:v>
+        <x:v>官网 Contact 页需浏览器渲染后可见邮箱；BD优先 business@，branding@/marketing@ 作为合作或营销转接，help@/recruit@ 不作为商务首选。</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -9254,7 +9254,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1148c88ff1f44400"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37ca67e76be64f0d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10193,10 +10193,10 @@
         <x:v>Random Dice 系列、B.B.TAN、Wild Tamer；Supercent 生态相关。</x:v>
       </x:c>
       <x:c r="G20" s="4" t="str">
-        <x:v>未公开商务邮箱</x:v>
+        <x:v>business@111percent.net; branding@111percent.net; marketing@111percent.net</x:v>
       </x:c>
       <x:c r="H20" s="4" t="str">
-        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://111percent.net/en/contact/</x:v>
+        <x:v>官网 Contact 页需浏览器渲染后可见邮箱；BD优先 business@，branding@/marketing@ 作为合作或营销转接，help@/recruit@ 不作为商务首选。</x:v>
       </x:c>
       <x:c r="I20" s="4" t="str">
         <x:v>Official site lists mobile casual portfolio and company focus.</x:v>
@@ -10270,7 +10270,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0613d74db6cd4b6f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb0f9e9d0e8c94404"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11324,7 +11324,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb36f010631d49c4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R63d86e528b0e435c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11519,7 +11519,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71f018ae6f9b4526"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc68b70bf26b4e59"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14911,7 +14911,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf1d4ff15ff764e34"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc0d48c4ac104d3d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add Gravity email discovery
</commit_message>
<xml_diff>
--- a/contact/rihanfx/jp_kr_game_outreach_workbook.xlsx
+++ b/contact/rihanfx/jp_kr_game_outreach_workbook.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README_Summary" sheetId="1" r:id="R09dda58d969448ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Longlist_80" sheetId="2" r:id="R57335e9ab5664944"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top20_Playbook" sheetId="3" r:id="R89268a58c97d4a01"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoring_Model" sheetId="4" r:id="Rf27884b0fb914144"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outreach_Pipeline" sheetId="5" r:id="R0743e28e701b44d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Templates" sheetId="6" r:id="R67fa21db76b04499"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source_Registry" sheetId="7" r:id="Rd147b87409494327"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README_Summary" sheetId="1" r:id="R29ef5d070bb749c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Longlist_80" sheetId="2" r:id="R6623e8fa658f4dcb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top20_Playbook" sheetId="3" r:id="R66b842e84a3547b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoring_Model" sheetId="4" r:id="R99c56404520b4c20"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outreach_Pipeline" sheetId="5" r:id="R11abb3b1d0a94d5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Templates" sheetId="6" r:id="Rfb3dacdeee834cb8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source_Registry" sheetId="7" r:id="R9da4b82e1fda404f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5232,10 +5232,10 @@
         <x:v>Ragnarok IP mobile/PC global publishing; regional operations</x:v>
       </x:c>
       <x:c r="AH43" s="7" t="str">
-        <x:v>未公开商务邮箱</x:v>
+        <x:v>business@gravity.co.kr; gbg@gravity.co.kr</x:v>
       </x:c>
       <x:c r="AI43" s="7" t="str">
-        <x:v>未找到公开商务邮箱；建议使用官方联系入口：https://www.gravity.co.kr/en/company/contact.asp</x:v>
+        <x:v>官网 Global Network 页需浏览器渲染后可见韩国总部 business@；同页 mailto 公开海外业务支持 gbg@，BD优先 business@。</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
@@ -9254,7 +9254,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37ca67e76be64f0d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1bc47cec075d466c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10270,7 +10270,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb0f9e9d0e8c94404"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc2d5f8e8e4546ac"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11324,7 +11324,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R63d86e528b0e435c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R41ca124131544beb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11519,7 +11519,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc68b70bf26b4e59"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9cbf0439872848fd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14911,7 +14911,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc0d48c4ac104d3d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa4ec33fa77e448f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>